<commit_message>
Sync site-content skill (location research step, ten-borough URL map)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017vTfMo1gkAD778K6pSTUtw
</commit_message>
<xml_diff>
--- a/.claude/skills/site-content/assets/manchester-gutters-url-map.xlsx
+++ b/.claude/skills/site-content/assets/manchester-gutters-url-map.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internal HTML'!$A$1:$N$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internal HTML'!$A$1:$N$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N45"/>
+  <dimension ref="A1:N64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -717,7 +717,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>/gutter-cleaning/</t>
+          <t>/fascias-and-soffits/</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -740,15 +740,15 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Gutter Cleaning Manchester | Manchester Gutters</t>
+          <t>Fascias and Soffits Manchester | Manchester Gutters</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Gutter Cleaning Manchester</t>
+          <t>Fascias and Soffits Manchester</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -781,7 +781,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>/fascias-and-soffits/</t>
+          <t>/downpipes/</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -804,15 +804,15 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Fascias and Soffits Manchester | Manchester Gutters</t>
+          <t>Downpipe Repairs Manchester | Manchester Gutters</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Fascias and Soffits Manchester</t>
+          <t>Downpipe Repairs Manchester</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -845,7 +845,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>/downpipes/</t>
+          <t>/gutter-cleaning/</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -868,15 +868,15 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Downpipe Repairs Manchester | Manchester Gutters</t>
+          <t>Gutter Cleaning Manchester | Manchester Gutters</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Downpipe Repairs Manchester</t>
+          <t>Gutter Cleaning Manchester</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -904,7 +904,11 @@
           <t>Service, WebPage, Person, FAQPage, BreadcrumbList</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Offered but not a priority (low-ticket). One page; left out of the location ranking and of hub and town priorities</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -970,7 +974,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Secondary trade: build only if roofing is in scope; it then needs its own hub named for the search</t>
+          <t>Secondary trade. The site is gutter-led by choice: gutters are easier to compete for and gutter jobs lead on to roofing. One service page if roofing is in scope; no roofing hubs</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1040,11 @@
           <t>WebPage, Service (areaServed), Person, BreadcrumbList, FAQPage</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>470 gutter searches a month</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1059,7 +1067,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>With a place brief</t>
+          <t>Wave 2, with a place brief</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1100,12 +1108,16 @@
           <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2: 30 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>/guttering-manchester/chorlton/</t>
+          <t>/guttering-manchester/clayton/</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1123,20 +1135,20 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>With a place brief</t>
+          <t>Wave 2, with a place brief</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Guttering Chorlton, Manchester | Manchester Gutters</t>
+          <t>Guttering Clayton, Manchester | Manchester Gutters</t>
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Guttering Chorlton, Manchester</t>
+          <t>Guttering Clayton, Manchester</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1164,21 +1176,25 @@
           <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2: 20 roofing searches a month (no gutter volume below hub level; roofing is the proxy); name also used elsewhere in the UK</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>/guttering-manchester/withington/</t>
+          <t>/guttering-stockport/</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Town</t>
+          <t>Area hub</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
@@ -1187,53 +1203,57 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>With a place brief</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Guttering Withington, Manchester | Manchester Gutters</t>
+          <t>Guttering Stockport | Repairs, Prices | Manchester Gutters</t>
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Guttering Withington, Manchester</t>
+          <t>Guttering Stockport</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>1,200-1,800</t>
+          <t>2,500-5,000</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
+          <t>Hero; credentials + logos; at a glance; what you need to know + office + form; town cards; services + problems we fix; costs table; projects/reviews/videos if records; why us; guide cards; FAQ 8-12; other hubs; CTA + form</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>its hub; nearest in-hub siblings; articles about the place</t>
+          <t>home; its towns; other hubs; articles about the place</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
+          <t>every service; every town under it; other hubs; guide cards</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>160 gutter searches a month</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>/guttering-manchester/levenshulme/</t>
+          <t>/guttering-stockport/cheadle/</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1251,20 +1271,20 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>With a place brief</t>
+          <t>Launch, with a place brief</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Guttering Levenshulme, Manchester | Manchester Gutters</t>
+          <t>Guttering Cheadle, Stockport | Manchester Gutters</t>
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Guttering Levenshulme, Manchester</t>
+          <t>Guttering Cheadle, Stockport</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1292,12 +1312,16 @@
           <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>Launch: 90 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>/guttering-manchester/sale/</t>
+          <t>/guttering-stockport/bramhall/</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1315,20 +1339,20 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>With a place brief</t>
+          <t>Launch, with a place brief</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Guttering Sale, Manchester | Manchester Gutters</t>
+          <t>Guttering Bramhall, Stockport | Manchester Gutters</t>
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Guttering Sale, Manchester</t>
+          <t>Guttering Bramhall, Stockport</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1356,12 +1380,16 @@
           <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>Launch: 50 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>/guttering-manchester/altrincham/</t>
+          <t>/guttering-stockport/cheadle-hulme/</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1379,20 +1407,20 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>With a place brief</t>
+          <t>Wave 2, with a place brief</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Guttering Altrincham, Manchester | Manchester Gutters</t>
+          <t>Guttering Cheadle Hulme, Stockport | Manchester Gutters</t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Guttering Altrincham, Manchester</t>
+          <t>Guttering Cheadle Hulme, Stockport</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1420,12 +1448,16 @@
           <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2: 40 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>/guttering-manchester/stretford/</t>
+          <t>/guttering-stockport/marple/</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1443,20 +1475,20 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>With a place brief</t>
+          <t>Wave 2, with a place brief</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Guttering Stretford, Manchester | Manchester Gutters</t>
+          <t>Guttering Marple, Stockport | Manchester Gutters</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Guttering Stretford, Manchester</t>
+          <t>Guttering Marple, Stockport</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1484,21 +1516,25 @@
           <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2: 40 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>/guttering-salford/</t>
+          <t>/guttering-stockport/davenport/</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Area hub</t>
+          <t>Town</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -1507,62 +1543,66 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Wave 2, with a place brief</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Guttering Salford | Repairs, Prices | Manchester Gutters</t>
+          <t>Guttering Davenport, Stockport | Manchester Gutters</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Guttering Salford</t>
+          <t>Guttering Davenport, Stockport</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>2,500-5,000</t>
+          <t>1,200-1,800</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Hero; credentials + logos; at a glance; what you need to know + office + form; town cards; services + problems we fix; costs table; projects/reviews/videos if records; why us; guide cards; FAQ 8-12; other hubs; CTA + form</t>
+          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>home; its towns; other hubs; articles about the place</t>
+          <t>its hub; nearest in-hub siblings; articles about the place</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>every service; every town under it; other hubs; guide cards</t>
+          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>WebPage, Service (areaServed), Person, BreadcrumbList, FAQPage</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2: 20 roofing searches a month (no gutter volume below hub level; roofing is the proxy); name also used elsewhere in the UK</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>/guttering-salford/eccles/</t>
+          <t>/guttering-oldham/</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Town</t>
+          <t>Area hub</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
@@ -1571,53 +1611,57 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>With a place brief</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Guttering Eccles, Salford | Manchester Gutters</t>
+          <t>Guttering Oldham | Repairs, Prices | Manchester Gutters</t>
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Guttering Eccles, Salford</t>
+          <t>Guttering Oldham</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>1,200-1,800</t>
+          <t>2,500-5,000</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
+          <t>Hero; credentials + logos; at a glance; what you need to know + office + form; town cards; services + problems we fix; costs table; projects/reviews/videos if records; why us; guide cards; FAQ 8-12; other hubs; CTA + form</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>its hub; nearest in-hub siblings; articles about the place</t>
+          <t>home; its towns; other hubs; articles about the place</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
+          <t>every service; every town under it; other hubs; guide cards</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>150 gutter searches a month</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>/guttering-salford/swinton/</t>
+          <t>/guttering-oldham/chadderton/</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1635,20 +1679,20 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>With a place brief</t>
+          <t>Wave 2, with a place brief</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Guttering Swinton, Salford | Manchester Gutters</t>
+          <t>Guttering Chadderton, Oldham | Manchester Gutters</t>
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Guttering Swinton, Salford</t>
+          <t>Guttering Chadderton, Oldham</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1676,21 +1720,25 @@
           <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2: 30 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>/guttering-salford/worsley/</t>
+          <t>/guttering-wigan/</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Town</t>
+          <t>Area hub</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -1699,62 +1747,66 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>With a place brief</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Guttering Worsley, Salford | Manchester Gutters</t>
+          <t>Guttering Wigan | Repairs, Prices | Manchester Gutters</t>
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Guttering Worsley, Salford</t>
+          <t>Guttering Wigan</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>1,200-1,800</t>
+          <t>2,500-5,000</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
+          <t>Hero; credentials + logos; at a glance; what you need to know + office + form; town cards; services + problems we fix; costs table; projects/reviews/videos if records; why us; guide cards; FAQ 8-12; other hubs; CTA + form</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>its hub; nearest in-hub siblings; articles about the place</t>
+          <t>home; its towns; other hubs; articles about the place</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
+          <t>every service; every town under it; other hubs; guide cards</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
-        </is>
-      </c>
-      <c r="N20" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>130 gutter searches a month</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>/guttering-stockport/</t>
+          <t>/guttering-wigan/leigh/</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Area hub</t>
+          <t>Town</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
@@ -1763,53 +1815,57 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Launch, with a place brief</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Guttering Stockport | Repairs, Prices | Manchester Gutters</t>
+          <t>Guttering Leigh, Wigan | Manchester Gutters</t>
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Guttering Stockport</t>
+          <t>Guttering Leigh, Wigan</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>2,500-5,000</t>
+          <t>1,200-1,800</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Hero; credentials + logos; at a glance; what you need to know + office + form; town cards; services + problems we fix; costs table; projects/reviews/videos if records; why us; guide cards; FAQ 8-12; other hubs; CTA + form</t>
+          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>home; its towns; other hubs; articles about the place</t>
+          <t>its hub; nearest in-hub siblings; articles about the place</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>every service; every town under it; other hubs; guide cards</t>
+          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>WebPage, Service (areaServed), Person, BreadcrumbList, FAQPage</t>
-        </is>
-      </c>
-      <c r="N21" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>Launch: 100 roofing searches a month (no gutter volume below hub level; roofing is the proxy); name also used elsewhere in the UK</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>/guttering-stockport/bramhall/</t>
+          <t>/guttering-wigan/atherton/</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1827,20 +1883,20 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>With a place brief</t>
+          <t>Wave 2, with a place brief</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Guttering Bramhall, Stockport | Manchester Gutters</t>
+          <t>Guttering Atherton, Wigan | Manchester Gutters</t>
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Guttering Bramhall, Stockport</t>
+          <t>Guttering Atherton, Wigan</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1868,12 +1924,16 @@
           <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
         </is>
       </c>
-      <c r="N22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2: 30 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>/guttering-stockport/cheadle/</t>
+          <t>/guttering-wigan/standish/</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1891,20 +1951,20 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>With a place brief</t>
+          <t>Wave 2, with a place brief</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Guttering Cheadle, Stockport | Manchester Gutters</t>
+          <t>Guttering Standish, Wigan | Manchester Gutters</t>
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Guttering Cheadle, Stockport</t>
+          <t>Guttering Standish, Wigan</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1932,21 +1992,25 @@
           <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
         </is>
       </c>
-      <c r="N23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2: 30 roofing searches a month (no gutter volume below hub level; roofing is the proxy); name also used elsewhere in the UK</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>/guttering-stockport/marple/</t>
+          <t>/guttering-bolton/</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Town</t>
+          <t>Area hub</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
@@ -1955,62 +2019,66 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>With a place brief</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Guttering Marple, Stockport | Manchester Gutters</t>
+          <t>Guttering Bolton | Repairs, Prices | Manchester Gutters</t>
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Guttering Marple, Stockport</t>
+          <t>Guttering Bolton</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>1,200-1,800</t>
+          <t>2,500-5,000</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
+          <t>Hero; credentials + logos; at a glance; what you need to know + office + form; town cards; services + problems we fix; costs table; projects/reviews/videos if records; why us; guide cards; FAQ 8-12; other hubs; CTA + form</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>its hub; nearest in-hub siblings; articles about the place</t>
+          <t>home; its towns; other hubs; articles about the place</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
+          <t>every service; every town under it; other hubs; guide cards</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
-        </is>
-      </c>
-      <c r="N24" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>120 gutter searches a month</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>/guttering-bolton/</t>
+          <t>/guttering-bolton/westhoughton/</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Area hub</t>
+          <t>Town</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
@@ -2019,48 +2087,52 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Wave 2, with a place brief</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Guttering Bolton | Repairs, Prices | Manchester Gutters</t>
+          <t>Guttering Westhoughton, Bolton | Manchester Gutters</t>
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Guttering Bolton</t>
+          <t>Guttering Westhoughton, Bolton</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>2,500-5,000</t>
+          <t>1,200-1,800</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Hero; credentials + logos; at a glance; what you need to know + office + form; town cards; services + problems we fix; costs table; projects/reviews/videos if records; why us; guide cards; FAQ 8-12; other hubs; CTA + form</t>
+          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>home; its towns; other hubs; articles about the place</t>
+          <t>its hub; nearest in-hub siblings; articles about the place</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>every service; every town under it; other hubs; guide cards</t>
+          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>WebPage, Service (areaServed), Person, BreadcrumbList, FAQPage</t>
-        </is>
-      </c>
-      <c r="N25" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2: 20 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2083,7 +2155,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>With a place brief</t>
+          <t>Wave 2, with a place brief</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -2124,21 +2196,25 @@
           <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
         </is>
       </c>
-      <c r="N26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2: 20 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>/guttering-bolton/farnworth/</t>
+          <t>/guttering-bury/</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Town</t>
+          <t>Area hub</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
@@ -2147,53 +2223,57 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>With a place brief</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Guttering Farnworth, Bolton | Manchester Gutters</t>
+          <t>Guttering Bury | Repairs, Prices | Manchester Gutters</t>
         </is>
       </c>
       <c r="G27" s="2" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Guttering Farnworth, Bolton</t>
+          <t>Guttering Bury</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>1,200-1,800</t>
+          <t>2,500-5,000</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
+          <t>Hero; credentials + logos; at a glance; what you need to know + office + form; town cards; services + problems we fix; costs table; projects/reviews/videos if records; why us; guide cards; FAQ 8-12; other hubs; CTA + form</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>its hub; nearest in-hub siblings; articles about the place</t>
+          <t>home; its towns; other hubs; articles about the place</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
+          <t>every service; every town under it; other hubs; guide cards</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
-        </is>
-      </c>
-      <c r="N27" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>70 gutter searches a month</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>/guttering-bolton/westhoughton/</t>
+          <t>/guttering-bury/prestwich/</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -2211,20 +2291,20 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>With a place brief</t>
+          <t>Launch, with a place brief</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Guttering Westhoughton, Bolton | Manchester Gutters</t>
+          <t>Guttering Prestwich, Bury | Manchester Gutters</t>
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Guttering Westhoughton, Bolton</t>
+          <t>Guttering Prestwich, Bury</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -2252,17 +2332,21 @@
           <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
         </is>
       </c>
-      <c r="N28" s="2" t="inlineStr"/>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>Launch: 60 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>/gutter-replacement/stockport/</t>
+          <t>/guttering-bury/ramsbottom/</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Service in place</t>
+          <t>Town</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2275,66 +2359,66 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Only with data</t>
+          <t>Wave 2, with a place brief</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Gutter Replacement Stockport | Manchester Gutters</t>
+          <t>Guttering Ramsbottom, Bury | Manchester Gutters</t>
         </is>
       </c>
       <c r="G29" s="2" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Gutter Replacement Stockport</t>
+          <t>Guttering Ramsbottom, Bury</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>1,200-2,200</t>
+          <t>1,200-1,800</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Mirror of the hub for one service</t>
+          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>its service; sibling cities</t>
+          <t>its hub; nearest in-hub siblings; articles about the place</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>up to the service; sibling cities; areas as text</t>
+          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Service (areaServed), WebPage, BreadcrumbList, FAQPage</t>
+          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>Built only when Search Console shows "&lt;service&gt; &lt;place&gt;" impressions with no page named for them</t>
+          <t>Wave 2: 30 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>/blog/gutter-repair-cost/</t>
+          <t>/guttering-rochdale/</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Article: pillar</t>
+          <t>Area hub</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
@@ -2343,58 +2427,62 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>With demand evidence</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>How Much Do Gutter Repairs Cost? | Manchester Gutters</t>
+          <t>Guttering Rochdale | Repairs, Prices | Manchester Gutters</t>
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>How Much Do Gutter Repairs Cost?</t>
+          <t>Guttering Rochdale</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>1,000-1,800</t>
+          <t>2,500-5,000</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; Read next; question H2s (60%+) with cost list, chart and comparison table; case/review/video if records; who to hire; guarantees; nearby areas; FAQ 10-12; related cards; CTA + form</t>
+          <t>Hero; credentials + logos; at a glance; what you need to know + office + form; town cards; services + problems we fix; costs table; projects/reviews/videos if records; why us; guide cards; FAQ 8-12; other hubs; CTA + form</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>blog index; hub guide cards; pillar/spokes</t>
+          <t>home; its towns; other hubs; articles about the place</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>services (3-5 in prose); the place hub and town; pillar once; Read next 3-4</t>
+          <t>every service; every town under it; other hubs; guide cards</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>BlogPosting, BreadcrumbList, FAQPage</t>
-        </is>
-      </c>
-      <c r="N30" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>60 gutter searches a month</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>/blog/gutter-repair-cost-manchester/</t>
+          <t>/guttering-rochdale/middleton/</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Article: spoke</t>
+          <t>Town</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2407,58 +2495,62 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>With demand evidence</t>
+          <t>Launch, with a place brief</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Gutter Repair Cost in Manchester | Manchester Gutters</t>
+          <t>Guttering Middleton, Rochdale | Manchester Gutters</t>
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Gutter Repair Cost in Manchester</t>
+          <t>Guttering Middleton, Rochdale</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>1,000-1,800</t>
+          <t>1,200-1,800</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; Read next; question H2s (60%+) with cost list, chart and comparison table; case/review/video if records; who to hire; guarantees; nearby areas; FAQ 10-12; related cards; CTA + form</t>
+          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>blog index; hub guide cards; pillar/spokes</t>
+          <t>its hub; nearest in-hub siblings; articles about the place</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>services (3-5 in prose); the place hub and town; pillar once; Read next 3-4</t>
+          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>BlogPosting, BreadcrumbList, FAQPage</t>
-        </is>
-      </c>
-      <c r="N31" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>Launch: 50 roofing searches a month (no gutter volume below hub level; roofing is the proxy); name also used elsewhere in the UK</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>/blog/gutter-cleaning-cost-stockport/</t>
+          <t>/guttering-rochdale/littleborough/</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Article: spoke</t>
+          <t>Town</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2471,12 +2563,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>With demand evidence</t>
+          <t>Wave 2, with a place brief</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Gutter Cleaning Cost in Stockport | Manchester Gutters</t>
+          <t>Guttering Littleborough, Rochdale | Manchester Gutters</t>
         </is>
       </c>
       <c r="G32" s="2" t="n">
@@ -2484,49 +2576,53 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Gutter Cleaning Cost in Stockport</t>
+          <t>Guttering Littleborough, Rochdale</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>1,000-1,800</t>
+          <t>1,200-1,800</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; Read next; question H2s (60%+) with cost list, chart and comparison table; case/review/video if records; who to hire; guarantees; nearby areas; FAQ 10-12; related cards; CTA + form</t>
+          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>blog index; hub guide cards; pillar/spokes</t>
+          <t>its hub; nearest in-hub siblings; articles about the place</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>services (3-5 in prose); the place hub and town; pillar once; Read next 3-4</t>
+          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>BlogPosting, BreadcrumbList, FAQPage</t>
-        </is>
-      </c>
-      <c r="N32" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2: 20 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>/blog/</t>
+          <t>/guttering-rochdale/langley/</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Blog index</t>
+          <t>Town</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
@@ -2535,58 +2631,62 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>When articles exist</t>
+          <t>Wave 2, with a place brief</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Guttering Guides and Costs | Manchester Gutters</t>
+          <t>Guttering Langley, Rochdale | Manchester Gutters</t>
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Guttering guides</t>
+          <t>Guttering Langley, Rochdale</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>200-400</t>
+          <t>1,200-1,800</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Groups by topic; 20 cards then pages</t>
+          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>nav</t>
+          <t>its hub; nearest in-hub siblings; articles about the place</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>every article</t>
+          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>CollectionPage, BreadcrumbList</t>
-        </is>
-      </c>
-      <c r="N33" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2: 20 roofing searches a month (no gutter volume below hub level; roofing is the proxy); name also used elsewhere in the UK</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>/reviews/</t>
+          <t>/guttering-salford/</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Proof</t>
+          <t>Area hub</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2599,62 +2699,66 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>When records exist</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Manchester Gutters Reviews and Ratings</t>
+          <t>Guttering Salford | Repairs, Prices | Manchester Gutters</t>
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Manchester Gutters Reviews and Ratings</t>
+          <t>Guttering Salford</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>as records allow</t>
+          <t>2,500-5,000</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+          <t>Hero; credentials + logos; at a glance; what you need to know + office + form; town cards; services + problems we fix; costs table; projects/reviews/videos if records; why us; guide cards; FAQ 8-12; other hubs; CTA + form</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>nav; footer; towns and services (1 in prose)</t>
+          <t>home; its towns; other hubs; articles about the place</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>issuers (Google profile, memberships)</t>
+          <t>every service; every town under it; other hubs; guide cards</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
-        </is>
-      </c>
-      <c r="N34" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>10 gutter searches a month; kept as the parent of its towns, no gutter demand under its own name</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>/case-studies/</t>
+          <t>/guttering-salford/swinton/</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Proof</t>
+          <t>Town</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
@@ -2663,62 +2767,66 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>When records exist</t>
+          <t>Wave 2, with a place brief</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Case Studies | Manchester Gutters</t>
+          <t>Guttering Swinton, Salford | Manchester Gutters</t>
         </is>
       </c>
       <c r="G35" s="2" t="n">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Case Studies</t>
+          <t>Guttering Swinton, Salford</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>as records allow</t>
+          <t>1,200-1,800</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>nav; footer; towns and services (1 in prose)</t>
+          <t>its hub; nearest in-hub siblings; articles about the place</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>issuers (Google profile, memberships)</t>
+          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
-        </is>
-      </c>
-      <c r="N35" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2: 40 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>/price-guide/</t>
+          <t>/guttering-salford/eccles/</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Proof</t>
+          <t>Town</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
@@ -2727,58 +2835,62 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>When records exist</t>
+          <t>Wave 2, with a place brief</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Guttering Price Guide | Manchester Gutters</t>
+          <t>Guttering Eccles, Salford | Manchester Gutters</t>
         </is>
       </c>
       <c r="G36" s="2" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Guttering Price Guide</t>
+          <t>Guttering Eccles, Salford</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>as records allow</t>
+          <t>1,200-1,800</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>nav; footer; towns and services (1 in prose)</t>
+          <t>its hub; nearest in-hub siblings; articles about the place</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>issuers (Google profile, memberships)</t>
+          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
-        </is>
-      </c>
-      <c r="N36" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2: 20 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>/gallery/</t>
+          <t>/guttering-tameside/</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Proof</t>
+          <t>Area hub</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2791,62 +2903,66 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>When records exist</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Gallery of Recent Jobs | Manchester Gutters</t>
+          <t>Guttering Tameside | Repairs, Prices | Manchester Gutters</t>
         </is>
       </c>
       <c r="G37" s="2" t="n">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Gallery of Recent Jobs</t>
+          <t>Guttering Tameside</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>as records allow</t>
+          <t>2,500-5,000</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+          <t>Hero; credentials + logos; at a glance; what you need to know + office + form; town cards; services + problems we fix; costs table; projects/reviews/videos if records; why us; guide cards; FAQ 8-12; other hubs; CTA + form</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>nav; footer; towns and services (1 in prose)</t>
+          <t>home; its towns; other hubs; articles about the place</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>issuers (Google profile, memberships)</t>
+          <t>every service; every town under it; other hubs; guide cards</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
-        </is>
-      </c>
-      <c r="N37" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>10 gutter searches a month; kept as the parent of its towns, no gutter demand under its own name</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>/about/</t>
+          <t>/guttering-tameside/denton/</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Company</t>
+          <t>Town</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
@@ -2855,12 +2971,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Launch, with a place brief</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>About Manchester Gutters | Local Guttering Team</t>
+          <t>Guttering Denton, Tameside | Manchester Gutters</t>
         </is>
       </c>
       <c r="G38" s="2" t="n">
@@ -2868,49 +2984,53 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>About Manchester Gutters</t>
+          <t>Guttering Denton, Tameside</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>600-1,200</t>
+          <t>1,200-1,800</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>Named people, credentials table, contact by area, map after consent</t>
+          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>nav; footer</t>
+          <t>its hub; nearest in-hub siblings; articles about the place</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>nav only</t>
+          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>AboutPage / ContactPage + Organization reference</t>
-        </is>
-      </c>
-      <c r="N38" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>Launch: 100 roofing searches a month (no gutter volume below hub level; roofing is the proxy); name also used elsewhere in the UK</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>/contact/</t>
+          <t>/guttering-tameside/ashton-under-lyne/</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Company</t>
+          <t>Town</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
@@ -2919,62 +3039,66 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Launch, with a place brief</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Contact Manchester Gutters | Free Guttering Quotes</t>
+          <t>Guttering Ashton-under-Lyne, Tameside | Manchester Gutters</t>
         </is>
       </c>
       <c r="G39" s="2" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Contact Manchester Gutters</t>
+          <t>Guttering Ashton-under-Lyne, Tameside</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>600-1,200</t>
+          <t>1,200-1,800</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>Named people, credentials table, contact by area, map after consent</t>
+          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>nav; footer</t>
+          <t>its hub; nearest in-hub siblings; articles about the place</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>nav only</t>
+          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>AboutPage / ContactPage + Organization reference</t>
-        </is>
-      </c>
-      <c r="N39" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>Launch: 50 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>/privacy-policy/</t>
+          <t>/guttering-tameside/hyde/</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Town</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
@@ -2983,62 +3107,66 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Wave 2, with a place brief</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Privacy Policy | Manchester Gutters</t>
+          <t>Guttering Hyde, Tameside | Manchester Gutters</t>
         </is>
       </c>
       <c r="G40" s="2" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Privacy Policy</t>
+          <t>Guttering Hyde, Tameside</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>as needed</t>
+          <t>1,200-1,800</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>What the site really does</t>
+          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>nav; footer</t>
+          <t>its hub; nearest in-hub siblings; articles about the place</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>nav only</t>
+          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>WebPage</t>
-        </is>
-      </c>
-      <c r="N40" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2: 30 roofing searches a month (no gutter volume below hub level; roofing is the proxy); name also used elsewhere in the UK</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>/cookie-policy/</t>
+          <t>/guttering-tameside/stalybridge/</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Town</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
@@ -3047,68 +3175,70 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Wave 2, with a place brief</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Cookie Policy | Manchester Gutters</t>
+          <t>Guttering Stalybridge, Tameside | Manchester Gutters</t>
         </is>
       </c>
       <c r="G41" s="2" t="n">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Cookie Policy</t>
+          <t>Guttering Stalybridge, Tameside</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>as needed</t>
+          <t>1,200-1,800</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>What the site really does</t>
+          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>nav; footer</t>
+          <t>its hub; nearest in-hub siblings; articles about the place</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>nav only</t>
+          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
         </is>
       </c>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>WebPage</t>
-        </is>
-      </c>
-      <c r="N41" s="2" t="inlineStr"/>
+          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2: 30 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>/404</t>
+          <t>/guttering-trafford/</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Utility</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+          <t>Area hub</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Non-indexable</t>
+          <t>Indexable</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -3118,260 +3248,1506 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Guttering Trafford | Repairs, Prices | Manchester Gutters</t>
         </is>
       </c>
       <c r="G42" s="2" t="n">
-        <v>1</v>
+        <v>57</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Guttering Trafford</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>2,500-5,000</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Hero; credentials + logos; at a glance; what you need to know + office + form; town cards; services + problems we fix; costs table; projects/reviews/videos if records; why us; guide cards; FAQ 8-12; other hubs; CTA + form</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>home; its towns; other hubs; articles about the place</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>every service; every town under it; other hubs; guide cards</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>WebPage, Service (areaServed), Person, BreadcrumbList, FAQPage</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>served with HTTP status 404</t>
+          <t>0 gutter searches a month; kept as the parent of its towns, no gutter demand under its own name</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>/sitemap.xml</t>
+          <t>/guttering-trafford/altrincham/</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Utility</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+          <t>Town</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Non-indexable</t>
+          <t>Indexable</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Launch, with a place brief</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Guttering Altrincham, Trafford | Manchester Gutters</t>
         </is>
       </c>
       <c r="G43" s="2" t="n">
-        <v>1</v>
+        <v>51</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Guttering Altrincham, Trafford</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>1,200-1,800</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>its hub; nearest in-hub siblings; articles about the place</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
         </is>
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>indexable pages only; real lastmod dates</t>
+          <t>Launch: 530 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>/robots.txt</t>
+          <t>/guttering-trafford/sale/</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Utility</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+          <t>Town</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Non-indexable</t>
+          <t>Indexable</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Launch, with a place brief</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Guttering Sale, Trafford | Manchester Gutters</t>
         </is>
       </c>
       <c r="G44" s="2" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Guttering Sale, Trafford</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>1,200-1,800</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>its hub; nearest in-hub siblings; articles about the place</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
         </is>
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>allows the AI search crawlers; points to the sitemap</t>
+          <t>Launch: 330 roofing searches a month (no gutter volume below hub level; roofing is the proxy); name also used elsewhere in the UK</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
+          <t>/guttering-trafford/urmston/</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Town</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Launch, with a place brief</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Guttering Urmston, Trafford | Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Guttering Urmston, Trafford</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>1,200-1,800</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>its hub; nearest in-hub siblings; articles about the place</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>Launch: 80 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>/guttering-trafford/hale/</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Town</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2, with a place brief</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Guttering Hale, Trafford | Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Guttering Hale, Trafford</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>1,200-1,800</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>its hub; nearest in-hub siblings; articles about the place</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2: 30 roofing searches a month (no gutter volume below hub level; roofing is the proxy); name also used elsewhere in the UK</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>/guttering-trafford/stretford/</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Town</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2, with a place brief</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Guttering Stretford, Trafford | Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Guttering Stretford, Trafford</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>1,200-1,800</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>Hero + breadcrumb; credentials; at a glance; local team + map; {Town} weather (3 H3); property types (3-4 H3); services grid; costings table; work in town if records; FAQ 6-8; nearby areas; CTA + form</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>its hub; nearest in-hub siblings; articles about the place</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>every service; its hub; 10-30 nearest siblings; proof (1 in prose)</t>
+        </is>
+      </c>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>WebPage, Service (areaServed = town), Person, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>Wave 2: 20 roofing searches a month (no gutter volume below hub level; roofing is the proxy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>/gutter-repairs/stockport/</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Service in place</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Only with data</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Gutter Repairs Stockport | Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Gutter Repairs Stockport</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>1,200-2,200</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Mirror of the hub for one service</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>its service; sibling cities</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>up to the service; sibling cities; areas as text</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>Service (areaServed), WebPage, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>Built only when Search Console shows "&lt;service&gt; &lt;place&gt;" impressions with no page named for them ("gutter repairs stockport": 110 a month in Keyword Planner)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>/blog/gutter-repair-cost/</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Article: pillar</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>With demand evidence</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>How Much Do Gutter Repairs Cost? | Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>How Much Do Gutter Repairs Cost?</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>1,000-1,800</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; Read next; question H2s (60%+) with cost list, chart and comparison table; case/review/video if records; who to hire; guarantees; nearby areas; FAQ 10-12; related cards; CTA + form</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>blog index; hub guide cards; pillar/spokes</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>services (3-5 in prose); the place hub and town; pillar once; Read next 3-4</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>BlogPosting, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>/blog/gutter-repair-cost-manchester/</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Article: spoke</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>With demand evidence</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Gutter Repair Cost in Manchester | Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Gutter Repair Cost in Manchester</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>1,000-1,800</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; Read next; question H2s (60%+) with cost list, chart and comparison table; case/review/video if records; who to hire; guarantees; nearby areas; FAQ 10-12; related cards; CTA + form</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>blog index; hub guide cards; pillar/spokes</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>services (3-5 in prose); the place hub and town; pillar once; Read next 3-4</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>BlogPosting, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>/blog/gutter-replacement-cost-stockport/</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Article: spoke</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>With demand evidence</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Gutter Replacement Cost in Stockport | Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Gutter Replacement Cost in Stockport</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>1,000-1,800</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; Read next; question H2s (60%+) with cost list, chart and comparison table; case/review/video if records; who to hire; guarantees; nearby areas; FAQ 10-12; related cards; CTA + form</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>blog index; hub guide cards; pillar/spokes</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>services (3-5 in prose); the place hub and town; pillar once; Read next 3-4</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>BlogPosting, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>/blog/</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Blog index</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>When articles exist</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Guttering Guides and Costs | Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Guttering guides</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>200-400</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>Groups by topic; 20 cards then pages</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>nav</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>every article</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>CollectionPage, BreadcrumbList</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>/reviews/</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Proof</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>When records exist</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Manchester Gutters Reviews and Ratings</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Manchester Gutters Reviews and Ratings</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>as records allow</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>nav; footer; towns and services (1 in prose)</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>issuers (Google profile, memberships)</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>/case-studies/</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Proof</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>When records exist</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Case Studies | Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Case Studies</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>as records allow</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>nav; footer; towns and services (1 in prose)</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>issuers (Google profile, memberships)</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>/price-guide/</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Proof</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>When records exist</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Guttering Price Guide | Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Guttering Price Guide</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>as records allow</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>nav; footer; towns and services (1 in prose)</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>issuers (Google profile, memberships)</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>/gallery/</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Proof</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>When records exist</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Gallery of Recent Jobs | Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Gallery of Recent Jobs</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>as records allow</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>nav; footer; towns and services (1 in prose)</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>issuers (Google profile, memberships)</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>/about/</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>About Manchester Gutters | Local Guttering Team</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>About Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>600-1,200</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>Named people, credentials table, contact by area, map after consent</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>nav; footer</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>nav only</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>AboutPage / ContactPage + Organization reference</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>/contact/</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Contact Manchester Gutters | Free Guttering Quotes</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Contact Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>600-1,200</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>Named people, credentials table, contact by area, map after consent</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>nav; footer</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>nav only</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>AboutPage / ContactPage + Organization reference</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>/privacy-policy/</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Privacy Policy | Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Privacy Policy</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>as needed</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>What the site really does</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>nav; footer</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>nav only</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>WebPage</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>/cookie-policy/</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Cookie Policy | Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Cookie Policy</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>as needed</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>What the site really does</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>nav; footer</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>nav only</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>WebPage</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>/404</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Non-indexable</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>served with HTTP status 404</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>/sitemap.xml</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Non-indexable</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>indexable pages only; real lastmod dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>/robots.txt</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Non-indexable</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>allows the AI search crawlers; points to the sitemap</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
           <t>/llms.txt</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>Utility</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>Non-indexable</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>Launch</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="G45" s="2" t="n">
+      <c r="G64" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="I64" s="2" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr">
+      <c r="J64" s="2" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="K45" s="2" t="inlineStr">
+      <c r="K64" s="2" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="L45" s="2" t="inlineStr">
+      <c r="L64" s="2" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="M45" s="2" t="inlineStr">
+      <c r="M64" s="2" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="N45" s="2" t="inlineStr">
+      <c r="N64" s="2" t="inlineStr">
         <is>
           <t>public facts only, from the facts file</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N45"/>
+  <autoFilter ref="A1:N64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3382,7 +4758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -3398,26 +4774,33 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Illustrative. Services, hubs and towns are confirmed by demand research (search volumes, top-10 overlap) and the client brief before anything is built.</t>
+          <t>Hubs and towns: from the location research ranking (Keyword Planner, UK, October 2026; manchester-gutters-location-research.xlsx). Hubs = the ten Greater Manchester boroughs; towns = Launch and Wave 2 rows. Hold towns stay in the ranking sheet.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Trade phrase in hub URLs is "guttering" pending the central-search-intent check; it may become "gutter-repairs" or "gutters".</t>
+          <t>Gutter-led by choice (Andrew, 25 October 2026). Gutter cleaning is offered but not a priority. Services and proof pages are confirmed by the client brief before anything is built.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Columns follow a Screaming Frog Internal: HTML export so the plan can be compared with a crawl of the built site.</t>
+          <t>Trade phrase in hub URLs is "guttering" pending the central-search-intent check; it may become "gutter-repairs" or "gutters".</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
+        <is>
+          <t>Columns follow a Screaming Frog Internal: HTML export so the plan can be compared with a crawl of the built site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Build stage: Launch = in the first release; With a place brief / With demand evidence / When records exist = added only when that condition is met.</t>
         </is>

</xml_diff>

<commit_message>
Sync site-content skill with audit-content (#619, #620)
Topic research from Search Console, Keyword Planner and Google autocomplete;
places from ONS wards and Wikidata; cost-article tables, contents list and
sources section on articles; the Manchester Gutters article plan.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017vTfMo1gkAD778K6pSTUtw
</commit_message>
<xml_diff>
--- a/.claude/skills/site-content/assets/manchester-gutters-url-map.xlsx
+++ b/.claude/skills/site-content/assets/manchester-gutters-url-map.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internal HTML'!$A$1:$N$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internal HTML'!$A$1:$N$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N64"/>
+  <dimension ref="A1:N75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -3701,7 +3701,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>/blog/gutter-repair-cost/</t>
+          <t>/blog/gutter-replacement-cost/</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -3719,20 +3719,20 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>With demand evidence</t>
+          <t>Launch, after the overlap test</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>How Much Do Gutter Repairs Cost? | Manchester Gutters</t>
+          <t>How Much Does Gutter Replacement Cost? | Manchester Gutters</t>
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>How Much Do Gutter Repairs Cost?</t>
+          <t>How Much Does Gutter Replacement Cost?</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
@@ -3742,17 +3742,17 @@
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; Read next; question H2s (60%+) with cost list, chart and comparison table; case/review/video if records; who to hire; guarantees; nearby areas; FAQ 10-12; related cards; CTA + form</t>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); three cost tables (by property type, additional costs, lifespan) from the client's records; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>blog index; hub guide cards; pillar/spokes</t>
+          <t>blog index; hub guide cards</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>services (3-5 in prose); the place hub and town; pillar once; Read next 3-4</t>
+          <t>services (3-5 in prose); the place hub; Read next 3-4; primary sources</t>
         </is>
       </c>
       <c r="M49" s="2" t="inlineStr">
@@ -3760,17 +3760,21 @@
           <t>BlogPosting, BreadcrumbList, FAQPage</t>
         </is>
       </c>
-      <c r="N49" s="2" t="inlineStr"/>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>3,640 UK searches a month across 21 searches (gutter replacement cost 1300; how much to replace guttering 390; new gutters price 320; how much do gutters cost 170). Folded in as sections: how long does guttering last, guttering building regulations, are gutter guards worth it, gutter guards cost. Sister site: Munster "how much to replace gutters" (234 impressions, position 5). Overlap test against /gutter-replacement/ before writing</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>/blog/gutter-repair-cost-manchester/</t>
+          <t>/blog/fascia-and-soffit-replacement-cost/</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Article: spoke</t>
+          <t>Article: pillar</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3783,20 +3787,20 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>With demand evidence</t>
+          <t>Launch, after the overlap test</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Gutter Repair Cost in Manchester | Manchester Gutters</t>
+          <t>Fascia and Soffit Replacement Cost | Manchester Gutters</t>
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Gutter Repair Cost in Manchester</t>
+          <t>Fascia and Soffit Replacement Cost</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
@@ -3806,17 +3810,17 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; Read next; question H2s (60%+) with cost list, chart and comparison table; case/review/video if records; who to hire; guarantees; nearby areas; FAQ 10-12; related cards; CTA + form</t>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); three cost tables (by property type, additional costs, lifespan) from the client's records; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>blog index; hub guide cards; pillar/spokes</t>
+          <t>blog index; hub guide cards</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>services (3-5 in prose); the place hub and town; pillar once; Read next 3-4</t>
+          <t>services (3-5 in prose); the place hub; Read next 3-4; primary sources</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr">
@@ -3824,17 +3828,21 @@
           <t>BlogPosting, BreadcrumbList, FAQPage</t>
         </is>
       </c>
-      <c r="N50" s="2" t="inlineStr"/>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>1,850 UK searches a month across 13 searches (cost of fascia and soffit replacement 590; soffit and fascia prices 390; fascia replacement cost 210; fascia board replacement cost 210). Folded in as sections: fascia capping vs replacement. Sister site: Munster fascia and soffit cost article: 57 clicks. Overlap test against /fascias-and-soffits/ before writing</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>/blog/gutter-replacement-cost-stockport/</t>
+          <t>/blog/roofline-replacement-cost/</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Article: spoke</t>
+          <t>Article: pillar</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3847,20 +3855,20 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>With demand evidence</t>
+          <t>Launch, after the overlap test</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Gutter Replacement Cost in Stockport | Manchester Gutters</t>
+          <t>Cost of New Gutters, Fascias and Soffits</t>
         </is>
       </c>
       <c r="G51" s="2" t="n">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Gutter Replacement Cost in Stockport</t>
+          <t>Cost of New Gutters, Fascias and Soffits</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
@@ -3870,17 +3878,17 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; Read next; question H2s (60%+) with cost list, chart and comparison table; case/review/video if records; who to hire; guarantees; nearby areas; FAQ 10-12; related cards; CTA + form</t>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); three cost tables (by property type, additional costs, lifespan) from the client's records; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>blog index; hub guide cards; pillar/spokes</t>
+          <t>blog index; hub guide cards</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>services (3-5 in prose); the place hub and town; pillar once; Read next 3-4</t>
+          <t>services (3-5 in prose); the place hub; Read next 3-4; primary sources</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
@@ -3888,21 +3896,25 @@
           <t>BlogPosting, BreadcrumbList, FAQPage</t>
         </is>
       </c>
-      <c r="N51" s="2" t="inlineStr"/>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>960 UK searches a month across 10 searches (gutter fascia and soffit replacement cost 320; gutter and fascia replacement cost 320; fascias and guttering cost 70; new gutter and fascia cost 50). Overlap test against /fascias-and-soffits/ and /gutter-replacement/ before writing</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>/blog/</t>
+          <t>/blog/gutter-repair-cost/</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Blog index</t>
+          <t>Article: pillar</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
@@ -3911,62 +3923,66 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>When articles exist</t>
+          <t>Launch, after the overlap test</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Guttering Guides and Costs | Manchester Gutters</t>
+          <t>How Much Do Gutter Repairs Cost? | Manchester Gutters</t>
         </is>
       </c>
       <c r="G52" s="2" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Guttering guides</t>
+          <t>How Much Do Gutter Repairs Cost?</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>200-400</t>
+          <t>1,000-1,800</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>Groups by topic; 20 cards then pages</t>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); three cost tables (by property type, additional costs, lifespan) from the client's records; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>nav</t>
+          <t>blog index; hub guide cards</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>every article</t>
+          <t>services (3-5 in prose); the place hub; Read next 3-4; primary sources</t>
         </is>
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>CollectionPage, BreadcrumbList</t>
-        </is>
-      </c>
-      <c r="N52" s="2" t="inlineStr"/>
+          <t>BlogPosting, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>640 UK searches a month across 8 searches (gutter repair cost 390; gutter leak repair cost 90; how much to repair gutters 50; leaking gutter repair cost 30). Sister site: Munster "Average cost of gutter repairs": 33 clicks. Overlap test against /gutter-repairs/ before writing</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>/reviews/</t>
+          <t>/blog/concrete-finlock-gutters/</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Proof</t>
+          <t>Article: pillar</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
@@ -3975,62 +3991,66 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>When records exist</t>
+          <t>Launch, after the overlap test</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Manchester Gutters Reviews and Ratings</t>
+          <t>Concrete Finlock Gutters, Repair or Replace</t>
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Manchester Gutters Reviews and Ratings</t>
+          <t>Concrete Finlock Gutters, Repair or Replace</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>as records allow</t>
+          <t>1,000-1,800</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); three cost tables (by property type, additional costs, lifespan) from the client's records; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>nav; footer; towns and services (1 in prose)</t>
+          <t>blog index; hub guide cards</t>
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>issuers (Google profile, memberships)</t>
+          <t>services (3-5 in prose); the place hub; Read next 3-4; primary sources</t>
         </is>
       </c>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
-        </is>
-      </c>
-      <c r="N53" s="2" t="inlineStr"/>
+          <t>BlogPosting, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr">
+        <is>
+          <t>240 UK searches a month across 4 searches (concrete gutter replacement cost 70; concrete gutter repair 70; finlock gutter removal cost 50; finlock gutter repair 50). Overlap test against /gutter-replacement/ before writing</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>/case-studies/</t>
+          <t>/blog/leaking-gutter-joint/</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Proof</t>
+          <t>Article: pillar</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
@@ -4039,62 +4059,66 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>When records exist</t>
+          <t>Launch, after the overlap test</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Case Studies | Manchester Gutters</t>
+          <t>How to Fix a Leaking Gutter Joint | Manchester Gutters</t>
         </is>
       </c>
       <c r="G54" s="2" t="n">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Case Studies</t>
+          <t>How to Fix a Leaking Gutter Joint</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>as records allow</t>
+          <t>1,000-1,800</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); comparison or step table; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>nav; footer; towns and services (1 in prose)</t>
+          <t>blog index; hub guide cards</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>issuers (Google profile, memberships)</t>
+          <t>services (3-5 in prose); the place hub; Read next 3-4; primary sources</t>
         </is>
       </c>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
-        </is>
-      </c>
-      <c r="N54" s="2" t="inlineStr"/>
+          <t>BlogPosting, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>2,100 UK searches a month across 10 searches (gutter leaking at joint 1000; sealing gutter joints 390; how to fix a leaking gutter joint 260; fix leaking gutter joint 170). Overlap test against /gutter-repairs/ before writing</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>/price-guide/</t>
+          <t>/blog/why-is-my-gutter-leaking/</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Proof</t>
+          <t>Article: pillar</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
@@ -4103,12 +4127,12 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>When records exist</t>
+          <t>Launch, after the overlap test</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Guttering Price Guide | Manchester Gutters</t>
+          <t>Why Is My Gutter Leaking and How to Fix It</t>
         </is>
       </c>
       <c r="G55" s="2" t="n">
@@ -4116,49 +4140,53 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Guttering Price Guide</t>
+          <t>Why Is My Gutter Leaking and How to Fix It</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>as records allow</t>
+          <t>1,000-1,800</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); comparison or step table; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>nav; footer; towns and services (1 in prose)</t>
+          <t>blog index; hub guide cards</t>
         </is>
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>issuers (Google profile, memberships)</t>
+          <t>services (3-5 in prose); the place hub; Read next 3-4; primary sources</t>
         </is>
       </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
-        </is>
-      </c>
-      <c r="N55" s="2" t="inlineStr"/>
+          <t>BlogPosting, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>1,520 UK searches a month across 10 searches (gutter leaking 480; gutter leak repairs 480; how to fix a leaking gutter 210; sealing gutter leaks 140). Overlap test against /gutter-repairs/ before writing</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>/gallery/</t>
+          <t>/blog/blocked-downpipe/</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Proof</t>
+          <t>Article: pillar</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
@@ -4167,62 +4195,66 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>When records exist</t>
+          <t>Launch, after the overlap test</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Gallery of Recent Jobs | Manchester Gutters</t>
+          <t>Blocked or Leaking Downpipe? What to Do | Manchester Gutters</t>
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Gallery of Recent Jobs</t>
+          <t>Blocked or Leaking Downpipe? What to Do</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>as records allow</t>
+          <t>1,000-1,800</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); comparison or step table; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>nav; footer; towns and services (1 in prose)</t>
+          <t>blog index; hub guide cards</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>issuers (Google profile, memberships)</t>
+          <t>services (3-5 in prose); the place hub; Read next 3-4; primary sources</t>
         </is>
       </c>
       <c r="M56" s="2" t="inlineStr">
         <is>
-          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
-        </is>
-      </c>
-      <c r="N56" s="2" t="inlineStr"/>
+          <t>BlogPosting, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>460 UK searches a month across 3 searches (downpipe blocked 260; how to unblock a downpipe 110; downpipe leaking 90). Overlap test against /downpipes/ before writing</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>/about/</t>
+          <t>/blog/rotten-fascia-boards/</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Company</t>
+          <t>Article: pillar</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
@@ -4231,62 +4263,66 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Launch, after the overlap test</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>About Manchester Gutters | Local Guttering Team</t>
+          <t>Rotten Fascia Boards, Repair or Replace?</t>
         </is>
       </c>
       <c r="G57" s="2" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>About Manchester Gutters</t>
+          <t>Rotten Fascia Boards, Repair or Replace?</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>600-1,200</t>
+          <t>1,000-1,800</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>Named people, credentials table, contact by area, map after consent</t>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); comparison or step table; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>nav; footer</t>
+          <t>blog index; hub guide cards</t>
         </is>
       </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>nav only</t>
+          <t>services (3-5 in prose); the place hub; Read next 3-4; primary sources</t>
         </is>
       </c>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>AboutPage / ContactPage + Organization reference</t>
-        </is>
-      </c>
-      <c r="N57" s="2" t="inlineStr"/>
+          <t>BlogPosting, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>420 UK searches a month across 4 searches (fixing soffits and fascias 170; how to fit fascia boards 140; rotten fascia boards 70; how to replace soffits 40). Folded in as sections: signs fascia needs replacing. Overlap test against /fascias-and-soffits/ before writing</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>/contact/</t>
+          <t>/blog/gutters-overflowing/</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Company</t>
+          <t>Article: pillar</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
@@ -4295,62 +4331,66 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Launch, after the overlap test</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Contact Manchester Gutters | Free Guttering Quotes</t>
+          <t>Why Are My Gutters Overflowing? | Manchester Gutters</t>
         </is>
       </c>
       <c r="G58" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Contact Manchester Gutters</t>
+          <t>Why Are My Gutters Overflowing?</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>600-1,200</t>
+          <t>1,000-1,800</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>Named people, credentials table, contact by area, map after consent</t>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); comparison or step table; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>nav; footer</t>
+          <t>blog index; hub guide cards</t>
         </is>
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>nav only</t>
+          <t>services (3-5 in prose); the place hub; Read next 3-4; primary sources</t>
         </is>
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>AboutPage / ContactPage + Organization reference</t>
-        </is>
-      </c>
-      <c r="N58" s="2" t="inlineStr"/>
+          <t>BlogPosting, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>340 UK searches a month across 3 searches (gutters overflowing 260; gutter overflowing in heavy rain 70; why are my gutters overflowing 10). Overlap test against /gutter-repairs/ before writing</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>/privacy-policy/</t>
+          <t>/blog/box-gutter-leaking/</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Article: pillar</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
@@ -4359,62 +4399,66 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Launch, after the overlap test</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Privacy Policy | Manchester Gutters</t>
+          <t>Leaking Box Gutters and Conservatory Gutters</t>
         </is>
       </c>
       <c r="G59" s="2" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Privacy Policy</t>
+          <t>Leaking Box Gutters and Conservatory Gutters</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>as needed</t>
+          <t>1,000-1,800</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>What the site really does</t>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); comparison or step table; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>nav; footer</t>
+          <t>blog index; hub guide cards</t>
         </is>
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>nav only</t>
+          <t>services (3-5 in prose); the place hub; Read next 3-4; primary sources</t>
         </is>
       </c>
       <c r="M59" s="2" t="inlineStr">
         <is>
-          <t>WebPage</t>
-        </is>
-      </c>
-      <c r="N59" s="2" t="inlineStr"/>
+          <t>BlogPosting, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="inlineStr">
+        <is>
+          <t>240 UK searches a month across 3 searches (conservatory box gutter leaking 140; fixing box gutters 70; box gutter leaking 30). Overlap test against /gutter-repairs/ before writing</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>/cookie-policy/</t>
+          <t>/blog/how-to-replace-guttering/</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Article: pillar</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
@@ -4423,208 +4467,206 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Launch, after the overlap test</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Cookie Policy | Manchester Gutters</t>
+          <t>How to Replace Guttering Step by Step | Manchester Gutters</t>
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Cookie Policy</t>
+          <t>How to Replace Guttering Step by Step</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>as needed</t>
+          <t>1,000-1,800</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>What the site really does</t>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); comparison or step table; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>nav; footer</t>
+          <t>blog index; hub guide cards</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>nav only</t>
+          <t>services (3-5 in prose); the place hub; Read next 3-4; primary sources</t>
         </is>
       </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>WebPage</t>
-        </is>
-      </c>
-      <c r="N60" s="2" t="inlineStr"/>
+          <t>BlogPosting, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>1,140 UK searches a month across 8 searches (how to replace guttering 480; how to fit guttering 210; how to fix guttering 170; how to cut guttering 170). Folded in as sections: tools for fitting guttering, gutter installation mistakes. Sister site: Munster step-by-step installation guide: 68 clicks. Overlap test against /gutter-replacement/ before writing</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>/404</t>
+          <t>/blog/gutter-fall-and-bracket-spacing/</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Utility</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+          <t>Article: pillar</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Non-indexable</t>
+          <t>Indexable</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Launch, after the overlap test</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Gutter Fall and Bracket Spacing Explained</t>
         </is>
       </c>
       <c r="G61" s="2" t="n">
-        <v>1</v>
+        <v>41</v>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Gutter Fall and Bracket Spacing Explained</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>1,000-1,800</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); comparison or step table; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>blog index; hub guide cards</t>
         </is>
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>services (3-5 in prose); the place hub; Read next 3-4; primary sources</t>
         </is>
       </c>
       <c r="M61" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>BlogPosting, BreadcrumbList, FAQPage</t>
         </is>
       </c>
       <c r="N61" s="2" t="inlineStr">
         <is>
-          <t>served with HTTP status 404</t>
+          <t>840 UK searches a month across 5 searches (fall for guttering 480; guttering fall per metre 140; how far apart should gutter brackets be 110; how many gutter brackets per meter 70). Overlap test against /gutter-replacement/ before writing</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>/sitemap.xml</t>
+          <t>/blog/rogue-roofers/</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Utility</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+          <t>Article: pillar</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Non-indexable</t>
+          <t>Indexable</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Launch, after the overlap test</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>How to Spot a Rogue Roofer and Hire Safely</t>
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>1</v>
+        <v>42</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>How to Spot a Rogue Roofer and Hire Safely</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>1,000-1,800</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); comparison or step table; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>blog index; hub guide cards</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>services (3-5 in prose); the place hub; Read next 3-4; primary sources</t>
         </is>
       </c>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>BlogPosting, BreadcrumbList, FAQPage</t>
         </is>
       </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>indexable pages only; real lastmod dates</t>
+          <t>280 UK searches a month across 6 searches (roofing scams 90; cowboy roofers 90; rogue roofers 40; roofing scams uk 30). Folded in as sections: how to complain about a builder. Sister site: Munster "Irish roofer scams": 72 clicks</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>/robots.txt</t>
+          <t>/blog/</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Utility</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+          <t>Blog index</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Non-indexable</t>
+          <t>Indexable</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -4634,120 +4676,838 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Guttering Guides and Costs | Manchester Gutters</t>
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Guttering guides</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>200-400</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Groups by topic; 20 cards then pages</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>nav</t>
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>every article</t>
         </is>
       </c>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N63" s="2" t="inlineStr">
-        <is>
-          <t>allows the AI search crawlers; points to the sitemap</t>
-        </is>
-      </c>
+          <t>CollectionPage, BreadcrumbList</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
+          <t>/reviews/</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Proof</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>When records exist</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Manchester Gutters Reviews and Ratings</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>Manchester Gutters Reviews and Ratings</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>as records allow</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>nav; footer; towns and services (1 in prose)</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>issuers (Google profile, memberships)</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>/case-studies/</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Proof</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>When records exist</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Case Studies | Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>Case Studies</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>as records allow</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>nav; footer; towns and services (1 in prose)</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>issuers (Google profile, memberships)</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
+        </is>
+      </c>
+      <c r="N65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>/price-guide/</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Proof</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>When records exist</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Guttering Price Guide | Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Guttering Price Guide</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>as records allow</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>nav; footer; towns and services (1 in prose)</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>issuers (Google profile, memberships)</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>/gallery/</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Proof</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>When records exist</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Gallery of Recent Jobs | Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>Gallery of Recent Jobs</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>as records allow</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>nav; footer; towns and services (1 in prose)</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>issuers (Google profile, memberships)</t>
+        </is>
+      </c>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>/about/</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>About Manchester Gutters | Local Guttering Team</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>About Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>600-1,200</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>Named people, credentials table, contact by area, map after consent</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>nav; footer</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>nav only</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>AboutPage / ContactPage + Organization reference</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>/contact/</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>Contact Manchester Gutters | Free Guttering Quotes</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>Contact Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>600-1,200</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>Named people, credentials table, contact by area, map after consent</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>nav; footer</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>nav only</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>AboutPage / ContactPage + Organization reference</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>/privacy-policy/</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Privacy Policy | Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Privacy Policy</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>as needed</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>What the site really does</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>nav; footer</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>nav only</t>
+        </is>
+      </c>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>WebPage</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>/cookie-policy/</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Indexable</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Cookie Policy | Manchester Gutters</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>Cookie Policy</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>as needed</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>What the site really does</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>nav; footer</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>nav only</t>
+        </is>
+      </c>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>WebPage</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>/404</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Non-indexable</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="inlineStr">
+        <is>
+          <t>served with HTTP status 404</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>/sitemap.xml</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Non-indexable</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr">
+        <is>
+          <t>indexable pages only; real lastmod dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>/robots.txt</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Non-indexable</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="inlineStr">
+        <is>
+          <t>allows the AI search crawlers; points to the sitemap</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
           <t>/llms.txt</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B75" s="2" t="inlineStr">
         <is>
           <t>Utility</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
+      <c r="C75" s="2" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="D75" s="2" t="inlineStr">
         <is>
           <t>Non-indexable</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="E75" s="2" t="inlineStr">
         <is>
           <t>Launch</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
+      <c r="F75" s="2" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="G64" s="2" t="n">
+      <c r="G75" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H64" s="2" t="inlineStr">
+      <c r="H75" s="2" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="I64" s="2" t="inlineStr">
+      <c r="I75" s="2" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="J64" s="2" t="inlineStr">
+      <c r="J75" s="2" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="K64" s="2" t="inlineStr">
+      <c r="K75" s="2" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="L64" s="2" t="inlineStr">
+      <c r="L75" s="2" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="M64" s="2" t="inlineStr">
+      <c r="M75" s="2" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="N64" s="2" t="inlineStr">
+      <c r="N75" s="2" t="inlineStr">
         <is>
           <t>public facts only, from the facts file</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N64"/>
+  <autoFilter ref="A1:N75"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Sync site-content skill with audit-content (#621)
Manchester Gutters article plan with autocomplete volumes: 16 articles.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017vTfMo1gkAD778K6pSTUtw
</commit_message>
<xml_diff>
--- a/.claude/skills/site-content/assets/manchester-gutters-url-map.xlsx
+++ b/.claude/skills/site-content/assets/manchester-gutters-url-map.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internal HTML'!$A$1:$N$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internal HTML'!$A$1:$N$77</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N75"/>
+  <dimension ref="A1:N77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -3762,7 +3762,7 @@
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>3,640 UK searches a month across 21 searches (gutter replacement cost 1300; how much to replace guttering 390; new gutters price 320; how much do gutters cost 170). Folded in as sections: how long does guttering last, guttering building regulations, are gutter guards worth it, gutter guards cost. Sister site: Munster "how much to replace gutters" (234 impressions, position 5). Overlap test against /gutter-replacement/ before writing</t>
+          <t>4,270 UK searches a month across 35 searches (gutter replacement cost 1300; how much to replace guttering 390; new gutters price 320; how much do gutters cost 170). Folded in as sections: how long does guttering last, guttering building regulations. Sister site: Munster "how much to replace gutters" (234 impressions, position 5). Overlap test against /gutter-replacement/ before writing</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3830,7 @@
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>1,850 UK searches a month across 13 searches (cost of fascia and soffit replacement 590; soffit and fascia prices 390; fascia replacement cost 210; fascia board replacement cost 210). Folded in as sections: fascia capping vs replacement. Sister site: Munster fascia and soffit cost article: 57 clicks. Overlap test against /fascias-and-soffits/ before writing</t>
+          <t>2,590 UK searches a month across 28 searches (cost of fascia and soffit replacement 590; soffit and fascia prices 390; fascia replacement cost 210; fascia board replacement cost 210). Folded in as sections: fascia capping vs replacement. Sister site: Munster fascia and soffit cost article: 57 clicks. Overlap test against /fascias-and-soffits/ before writing</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>640 UK searches a month across 8 searches (gutter repair cost 390; gutter leak repair cost 90; how much to repair gutters 50; leaking gutter repair cost 30). Sister site: Munster "Average cost of gutter repairs": 33 clicks. Overlap test against /gutter-repairs/ before writing</t>
+          <t>640 UK searches a month across 9 searches (gutter repair cost 390; gutter leak repair cost 90; how much to repair gutters 50; leaking gutter repair cost 30). Sister site: Munster "Average cost of gutter repairs": 33 clicks. Overlap test against /gutter-repairs/ before writing</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>/blog/leaking-gutter-joint/</t>
+          <t>/blog/what-are-fascias-and-soffits/</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -4064,15 +4064,15 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>How to Fix a Leaking Gutter Joint | Manchester Gutters</t>
+          <t>What Are Fascias and Soffits on a House?</t>
         </is>
       </c>
       <c r="G54" s="2" t="n">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>How to Fix a Leaking Gutter Joint</t>
+          <t>What Are Fascias and Soffits on a House?</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
@@ -4102,14 +4102,14 @@
       </c>
       <c r="N54" s="2" t="inlineStr">
         <is>
-          <t>2,100 UK searches a month across 10 searches (gutter leaking at joint 1000; sealing gutter joints 390; how to fix a leaking gutter joint 260; fix leaking gutter joint 170). Overlap test against /gutter-repairs/ before writing</t>
+          <t>4,120 UK searches a month across 19 searches (what are soffits and fascias 1300; what are fascias on a house 590; fascia vs soffit 320; what are soffits on a house 320). Overlap test against /fascias-and-soffits/ before writing</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>/blog/why-is-my-gutter-leaking/</t>
+          <t>/blog/leaking-gutter-joint/</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -4132,15 +4132,15 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Why Is My Gutter Leaking and How to Fix It</t>
+          <t>How to Fix a Leaking Gutter Joint | Manchester Gutters</t>
         </is>
       </c>
       <c r="G55" s="2" t="n">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Why Is My Gutter Leaking and How to Fix It</t>
+          <t>How to Fix a Leaking Gutter Joint</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
@@ -4170,14 +4170,14 @@
       </c>
       <c r="N55" s="2" t="inlineStr">
         <is>
-          <t>1,520 UK searches a month across 10 searches (gutter leaking 480; gutter leak repairs 480; how to fix a leaking gutter 210; sealing gutter leaks 140). Overlap test against /gutter-repairs/ before writing</t>
+          <t>2,410 UK searches a month across 16 searches (gutter leaking at joint 1000; sealing gutter joints 390; how to fix a leaking gutter joint 260; fix leaking gutter joint 170). Overlap test against /gutter-repairs/ before writing</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>/blog/blocked-downpipe/</t>
+          <t>/blog/why-is-my-gutter-leaking/</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -4200,15 +4200,15 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Blocked or Leaking Downpipe? What to Do | Manchester Gutters</t>
+          <t>Why Is My Gutter Leaking and How to Fix It</t>
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Blocked or Leaking Downpipe? What to Do</t>
+          <t>Why Is My Gutter Leaking and How to Fix It</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
@@ -4238,14 +4238,14 @@
       </c>
       <c r="N56" s="2" t="inlineStr">
         <is>
-          <t>460 UK searches a month across 3 searches (downpipe blocked 260; how to unblock a downpipe 110; downpipe leaking 90). Overlap test against /downpipes/ before writing</t>
+          <t>1,600 UK searches a month across 13 searches (gutter leaking 480; gutter leak repairs 480; how to fix a leaking gutter 210; sealing gutter leaks 140). Overlap test against /gutter-repairs/ before writing</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>/blog/rotten-fascia-boards/</t>
+          <t>/blog/blocked-downpipe/</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -4268,15 +4268,15 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Rotten Fascia Boards, Repair or Replace?</t>
+          <t>Blocked or Leaking Downpipe? What to Do | Manchester Gutters</t>
         </is>
       </c>
       <c r="G57" s="2" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Rotten Fascia Boards, Repair or Replace?</t>
+          <t>Blocked or Leaking Downpipe? What to Do</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
@@ -4306,14 +4306,14 @@
       </c>
       <c r="N57" s="2" t="inlineStr">
         <is>
-          <t>420 UK searches a month across 4 searches (fixing soffits and fascias 170; how to fit fascia boards 140; rotten fascia boards 70; how to replace soffits 40). Folded in as sections: signs fascia needs replacing. Overlap test against /fascias-and-soffits/ before writing</t>
+          <t>990 UK searches a month across 11 searches (downpipe blocked 260; blocked downpipe from gutter 210; how to unblock a downpipe 110; downpipe leaking 90). Overlap test against /downpipes/ before writing</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>/blog/gutters-overflowing/</t>
+          <t>/blog/rotten-fascia-boards/</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -4336,15 +4336,15 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Why Are My Gutters Overflowing? | Manchester Gutters</t>
+          <t>Rotten Fascia Boards, Repair or Replace?</t>
         </is>
       </c>
       <c r="G58" s="2" t="n">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Why Are My Gutters Overflowing?</t>
+          <t>Rotten Fascia Boards, Repair or Replace?</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
@@ -4374,7 +4374,7 @@
       </c>
       <c r="N58" s="2" t="inlineStr">
         <is>
-          <t>340 UK searches a month across 3 searches (gutters overflowing 260; gutter overflowing in heavy rain 70; why are my gutters overflowing 10). Overlap test against /gutter-repairs/ before writing</t>
+          <t>980 UK searches a month across 14 searches (fixing soffits and fascias 170; how to fit fascia boards 140; how to replace fascia and soffit 110; how to install fascia boards 90). Folded in as sections: signs fascia needs replacing. Overlap test against /fascias-and-soffits/ before writing</t>
         </is>
       </c>
     </row>
@@ -4442,14 +4442,14 @@
       </c>
       <c r="N59" s="2" t="inlineStr">
         <is>
-          <t>240 UK searches a month across 3 searches (conservatory box gutter leaking 140; fixing box gutters 70; box gutter leaking 30). Overlap test against /gutter-repairs/ before writing</t>
+          <t>380 UK searches a month across 5 searches (conservatory box gutter leaking 140; what are box gutters 90; fixing box gutters 70; box gutter sizes 50). Overlap test against /gutter-repairs/ before writing</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>/blog/how-to-replace-guttering/</t>
+          <t>/blog/gutters-overflowing/</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -4472,15 +4472,15 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>How to Replace Guttering Step by Step | Manchester Gutters</t>
+          <t>Why Are My Gutters Overflowing? | Manchester Gutters</t>
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>How to Replace Guttering Step by Step</t>
+          <t>Why Are My Gutters Overflowing?</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
@@ -4510,7 +4510,7 @@
       </c>
       <c r="N60" s="2" t="inlineStr">
         <is>
-          <t>1,140 UK searches a month across 8 searches (how to replace guttering 480; how to fit guttering 210; how to fix guttering 170; how to cut guttering 170). Folded in as sections: tools for fitting guttering, gutter installation mistakes. Sister site: Munster step-by-step installation guide: 68 clicks. Overlap test against /gutter-replacement/ before writing</t>
+          <t>340 UK searches a month across 3 searches (gutters overflowing 260; gutter overflowing in heavy rain 70; why are my gutters overflowing 10). Overlap test against /gutter-repairs/ before writing</t>
         </is>
       </c>
     </row>
@@ -4540,15 +4540,15 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Gutter Fall and Bracket Spacing Explained</t>
+          <t>Gutter Brackets and Fall Explained | Manchester Gutters</t>
         </is>
       </c>
       <c r="G61" s="2" t="n">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Gutter Fall and Bracket Spacing Explained</t>
+          <t>Gutter Brackets and Fall Explained</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
@@ -4578,14 +4578,14 @@
       </c>
       <c r="N61" s="2" t="inlineStr">
         <is>
-          <t>840 UK searches a month across 5 searches (fall for guttering 480; guttering fall per metre 140; how far apart should gutter brackets be 110; how many gutter brackets per meter 70). Overlap test against /gutter-replacement/ before writing</t>
+          <t>2,480 UK searches a month across 20 searches (gutter brackets rise and fall 590; fall for guttering 480; types of gutter brackets 170; guttering fall per metre 140). Overlap test against /gutter-replacement/ before writing</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>/blog/rogue-roofers/</t>
+          <t>/blog/how-to-replace-guttering/</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -4608,15 +4608,15 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>How to Spot a Rogue Roofer and Hire Safely</t>
+          <t>How to Replace Guttering Step by Step | Manchester Gutters</t>
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>How to Spot a Rogue Roofer and Hire Safely</t>
+          <t>How to Replace Guttering Step by Step</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
@@ -4646,23 +4646,23 @@
       </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>280 UK searches a month across 6 searches (roofing scams 90; cowboy roofers 90; rogue roofers 40; roofing scams uk 30). Folded in as sections: how to complain about a builder. Sister site: Munster "Irish roofer scams": 72 clicks</t>
+          <t>1,290 UK searches a month across 14 searches (how to replace guttering 480; how to fit guttering 210; how to fix guttering 170; how to cut guttering 170). Folded in as sections: tools for fitting guttering, gutter installation mistakes. Sister site: Munster step-by-step installation guide: 68 clicks. Overlap test against /gutter-replacement/ before writing</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>/blog/</t>
+          <t>/blog/are-gutter-guards-worth-it/</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Blog index</t>
+          <t>Article: pillar</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
@@ -4671,62 +4671,66 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Launch, after the overlap test</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Guttering Guides and Costs | Manchester Gutters</t>
+          <t>Gutter Guards, Are They Worth Fitting? | Manchester Gutters</t>
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Guttering guides</t>
+          <t>Gutter Guards, Are They Worth Fitting?</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>200-400</t>
+          <t>1,000-1,800</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>Groups by topic; 20 cards then pages</t>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); comparison or step table; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>nav</t>
+          <t>blog index; hub guide cards</t>
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>every article</t>
+          <t>services (3-5 in prose); the place hub; Read next 3-4; primary sources</t>
         </is>
       </c>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>CollectionPage, BreadcrumbList</t>
-        </is>
-      </c>
-      <c r="N63" s="2" t="inlineStr"/>
+          <t>BlogPosting, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>350 UK searches a month across 6 searches (best gutter guards 170; cost of gutter guards 50; are gutter guards worth it 40; what gutter guard is best 30). Overlap test against /gutter-replacement/ before writing</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>/reviews/</t>
+          <t>/blog/rogue-roofers/</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Proof</t>
+          <t>Article: pillar</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
@@ -4735,58 +4739,62 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>When records exist</t>
+          <t>Launch, after the overlap test</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Manchester Gutters Reviews and Ratings</t>
+          <t>How to Spot a Rogue Roofer and Hire Safely</t>
         </is>
       </c>
       <c r="G64" s="2" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Manchester Gutters Reviews and Ratings</t>
+          <t>How to Spot a Rogue Roofer and Hire Safely</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>as records allow</t>
+          <t>1,000-1,800</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); comparison or step table; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>nav; footer; towns and services (1 in prose)</t>
+          <t>blog index; hub guide cards</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>issuers (Google profile, memberships)</t>
+          <t>services (3-5 in prose); the place hub; Read next 3-4; primary sources</t>
         </is>
       </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
-        </is>
-      </c>
-      <c r="N64" s="2" t="inlineStr"/>
+          <t>BlogPosting, BreadcrumbList, FAQPage</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>280 UK searches a month across 6 searches (roofing scams 90; cowboy roofers 90; rogue roofers 40; roofing scams uk 30). Folded in as sections: how to complain about a builder. Sister site: Munster "Irish roofer scams": 72 clicks</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>/case-studies/</t>
+          <t>/blog/</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Proof</t>
+          <t>Blog index</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4799,45 +4807,45 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>When records exist</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Case Studies | Manchester Gutters</t>
+          <t>Guttering Guides and Costs | Manchester Gutters</t>
         </is>
       </c>
       <c r="G65" s="2" t="n">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Case Studies</t>
+          <t>Guttering guides</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>as records allow</t>
+          <t>200-400</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+          <t>Groups by topic; 20 cards then pages</t>
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>nav; footer; towns and services (1 in prose)</t>
+          <t>nav</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>issuers (Google profile, memberships)</t>
+          <t>every article</t>
         </is>
       </c>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
+          <t>CollectionPage, BreadcrumbList</t>
         </is>
       </c>
       <c r="N65" s="2" t="inlineStr"/>
@@ -4845,7 +4853,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>/price-guide/</t>
+          <t>/reviews/</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -4868,15 +4876,15 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Guttering Price Guide | Manchester Gutters</t>
+          <t>Manchester Gutters Reviews and Ratings</t>
         </is>
       </c>
       <c r="G66" s="2" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Guttering Price Guide</t>
+          <t>Manchester Gutters Reviews and Ratings</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -4909,7 +4917,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>/gallery/</t>
+          <t>/case-studies/</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -4932,15 +4940,15 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Gallery of Recent Jobs | Manchester Gutters</t>
+          <t>Case Studies | Manchester Gutters</t>
         </is>
       </c>
       <c r="G67" s="2" t="n">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Gallery of Recent Jobs</t>
+          <t>Case Studies</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -4973,12 +4981,12 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>/about/</t>
+          <t>/price-guide/</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Company</t>
+          <t>Proof</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4991,45 +4999,45 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>When records exist</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>About Manchester Gutters | Local Guttering Team</t>
+          <t>Guttering Price Guide | Manchester Gutters</t>
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>About Manchester Gutters</t>
+          <t>Guttering Price Guide</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>600-1,200</t>
+          <t>as records allow</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>Named people, credentials table, contact by area, map after consent</t>
+          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>nav; footer</t>
+          <t>nav; footer; towns and services (1 in prose)</t>
         </is>
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>nav only</t>
+          <t>issuers (Google profile, memberships)</t>
         </is>
       </c>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>AboutPage / ContactPage + Organization reference</t>
+          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
         </is>
       </c>
       <c r="N68" s="2" t="inlineStr"/>
@@ -5037,12 +5045,12 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>/contact/</t>
+          <t>/gallery/</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Company</t>
+          <t>Proof</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -5055,45 +5063,45 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>When records exist</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Contact Manchester Gutters | Free Guttering Quotes</t>
+          <t>Gallery of Recent Jobs | Manchester Gutters</t>
         </is>
       </c>
       <c r="G69" s="2" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>Contact Manchester Gutters</t>
+          <t>Gallery of Recent Jobs</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>600-1,200</t>
+          <t>as records allow</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>Named people, credentials table, contact by area, map after consent</t>
+          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>nav; footer</t>
+          <t>nav; footer; towns and services (1 in prose)</t>
         </is>
       </c>
       <c r="L69" s="2" t="inlineStr">
         <is>
-          <t>nav only</t>
+          <t>issuers (Google profile, memberships)</t>
         </is>
       </c>
       <c r="M69" s="2" t="inlineStr">
         <is>
-          <t>AboutPage / ContactPage + Organization reference</t>
+          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
         </is>
       </c>
       <c r="N69" s="2" t="inlineStr"/>
@@ -5101,12 +5109,12 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>/privacy-policy/</t>
+          <t>/about/</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Company</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -5124,25 +5132,25 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Privacy Policy | Manchester Gutters</t>
+          <t>About Manchester Gutters | Local Guttering Team</t>
         </is>
       </c>
       <c r="G70" s="2" t="n">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Privacy Policy</t>
+          <t>About Manchester Gutters</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>as needed</t>
+          <t>600-1,200</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>What the site really does</t>
+          <t>Named people, credentials table, contact by area, map after consent</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
@@ -5157,7 +5165,7 @@
       </c>
       <c r="M70" s="2" t="inlineStr">
         <is>
-          <t>WebPage</t>
+          <t>AboutPage / ContactPage + Organization reference</t>
         </is>
       </c>
       <c r="N70" s="2" t="inlineStr"/>
@@ -5165,12 +5173,12 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>/cookie-policy/</t>
+          <t>/contact/</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Company</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -5188,25 +5196,25 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Cookie Policy | Manchester Gutters</t>
+          <t>Contact Manchester Gutters | Free Guttering Quotes</t>
         </is>
       </c>
       <c r="G71" s="2" t="n">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Cookie Policy</t>
+          <t>Contact Manchester Gutters</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>as needed</t>
+          <t>600-1,200</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>What the site really does</t>
+          <t>Named people, credentials table, contact by area, map after consent</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr">
@@ -5221,7 +5229,7 @@
       </c>
       <c r="M71" s="2" t="inlineStr">
         <is>
-          <t>WebPage</t>
+          <t>AboutPage / ContactPage + Organization reference</t>
         </is>
       </c>
       <c r="N71" s="2" t="inlineStr"/>
@@ -5229,22 +5237,20 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>/404</t>
+          <t>/privacy-policy/</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Utility</t>
-        </is>
-      </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Non-indexable</t>
+          <t>Indexable</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -5254,67 +5260,61 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Privacy Policy | Manchester Gutters</t>
         </is>
       </c>
       <c r="G72" s="2" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Privacy Policy</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>as needed</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>What the site really does</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>nav; footer</t>
         </is>
       </c>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>nav only</t>
         </is>
       </c>
       <c r="M72" s="2" t="inlineStr">
         <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N72" s="2" t="inlineStr">
-        <is>
-          <t>served with HTTP status 404</t>
-        </is>
-      </c>
+          <t>WebPage</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>/sitemap.xml</t>
+          <t>/cookie-policy/</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Utility</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Non-indexable</t>
+          <t>Indexable</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -5324,52 +5324,48 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Cookie Policy | Manchester Gutters</t>
         </is>
       </c>
       <c r="G73" s="2" t="n">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Cookie Policy</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>as needed</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>What the site really does</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>nav; footer</t>
         </is>
       </c>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>nav only</t>
         </is>
       </c>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N73" s="2" t="inlineStr">
-        <is>
-          <t>indexable pages only; real lastmod dates</t>
-        </is>
-      </c>
+          <t>WebPage</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>/robots.txt</t>
+          <t>/404</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -5432,14 +5428,14 @@
       </c>
       <c r="N74" s="2" t="inlineStr">
         <is>
-          <t>allows the AI search crawlers; points to the sitemap</t>
+          <t>served with HTTP status 404</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>/llms.txt</t>
+          <t>/sitemap.xml</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -5502,12 +5498,152 @@
       </c>
       <c r="N75" s="2" t="inlineStr">
         <is>
+          <t>indexable pages only; real lastmod dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>/robots.txt</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Non-indexable</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="inlineStr">
+        <is>
+          <t>allows the AI search crawlers; points to the sitemap</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>/llms.txt</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Non-indexable</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L77" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N77" s="2" t="inlineStr">
+        <is>
           <t>public facts only, from the facts file</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N75"/>
+  <autoFilter ref="A1:N77"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: sync site-content skill after audit-content#625
Overlap test results for the Manchester article pairs, the roofline cost
article merged into the fascia and soffit cost article, the rebuilt URL map
and site tree, and how to run the overlap test (topic-research.md step 5).
Copy identical to audit-content master c2777b0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016DXh5ATFKvUL6hqSuDkrz5
</commit_message>
<xml_diff>
--- a/.claude/skills/site-content/assets/manchester-gutters-url-map.xlsx
+++ b/.claude/skills/site-content/assets/manchester-gutters-url-map.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internal HTML'!$A$1:$N$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internal HTML'!$A$1:$N$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N77"/>
+  <dimension ref="A1:N76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -3719,7 +3719,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Launch, after the overlap test</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -3762,7 +3762,7 @@
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>4,270 UK searches a month across 35 searches (gutter replacement cost 1300; how much to replace guttering 390; new gutters price 320; how much do gutters cost 170). Folded in as sections: how long does guttering last, guttering building regulations. Sister site: Munster "how much to replace gutters" (234 impressions, position 5). Overlap test against /gutter-replacement/ before writing</t>
+          <t>4,270 UK searches a month across 35 searches (gutter replacement cost 1300; how much to replace guttering 390; new gutters price 320; how much do gutters cost 170). Folded in as sections: how long does guttering last, guttering building regulations. Sister site: Munster "how much to replace gutters" (234 impressions, position 5). Overlap test passed: 20% vs "gutter replacement manchester" (/gutter-replacement/)</t>
         </is>
       </c>
     </row>
@@ -3787,7 +3787,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Launch, after the overlap test</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -3830,14 +3830,14 @@
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>2,590 UK searches a month across 28 searches (cost of fascia and soffit replacement 590; soffit and fascia prices 390; fascia replacement cost 210; fascia board replacement cost 210). Folded in as sections: fascia capping vs replacement. Sister site: Munster fascia and soffit cost article: 57 clicks. Overlap test against /fascias-and-soffits/ before writing</t>
+          <t>3,550 UK searches a month across 38 searches (cost of fascia and soffit replacement 590; soffit and fascia prices 390; gutter fascia and soffit replacement cost 320; gutter and fascia replacement cost 320). Folded in as sections: fascia capping vs replacement, gutters, fascias and soffits replaced together (from roofline-replacement-cost, 90% overlap). Sister site: Munster fascia and soffit cost article: 57 clicks. Overlap test passed: 10% vs "fascias and soffits manchester" (/fascias-and-soffits/); 40% vs "gutter replacement cost" (/blog/gutter-replacement-cost/)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>/blog/roofline-replacement-cost/</t>
+          <t>/blog/gutter-repair-cost/</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -3855,20 +3855,20 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Launch, after the overlap test</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Cost of New Gutters, Fascias and Soffits</t>
+          <t>How Much Do Gutter Repairs Cost? | Manchester Gutters</t>
         </is>
       </c>
       <c r="G51" s="2" t="n">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Cost of New Gutters, Fascias and Soffits</t>
+          <t>How Much Do Gutter Repairs Cost?</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
@@ -3898,14 +3898,14 @@
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>960 UK searches a month across 10 searches (gutter fascia and soffit replacement cost 320; gutter and fascia replacement cost 320; fascias and guttering cost 70; new gutter and fascia cost 50). Overlap test against /fascias-and-soffits/ and /gutter-replacement/ before writing</t>
+          <t>640 UK searches a month across 9 searches (gutter repair cost 390; gutter leak repair cost 90; how much to repair gutters 50; leaking gutter repair cost 30). Sister site: Munster "Average cost of gutter repairs": 33 clicks. Overlap test passed: 0% vs "gutter repairs manchester" (/gutter-repairs/)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>/blog/gutter-repair-cost/</t>
+          <t>/blog/concrete-finlock-gutters/</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -3928,15 +3928,15 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>How Much Do Gutter Repairs Cost? | Manchester Gutters</t>
+          <t>Concrete Finlock Gutters, Repair or Replace</t>
         </is>
       </c>
       <c r="G52" s="2" t="n">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>How Much Do Gutter Repairs Cost?</t>
+          <t>Concrete Finlock Gutters, Repair or Replace</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
@@ -3966,14 +3966,14 @@
       </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>640 UK searches a month across 9 searches (gutter repair cost 390; gutter leak repair cost 90; how much to repair gutters 50; leaking gutter repair cost 30). Sister site: Munster "Average cost of gutter repairs": 33 clicks. Overlap test against /gutter-repairs/ before writing</t>
+          <t>240 UK searches a month across 4 searches (concrete gutter replacement cost 70; concrete gutter repair 70; finlock gutter removal cost 50; finlock gutter repair 50). Overlap test against /gutter-replacement/ before writing</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>/blog/concrete-finlock-gutters/</t>
+          <t>/blog/what-are-fascias-and-soffits/</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -3991,20 +3991,20 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Launch, after the overlap test</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Concrete Finlock Gutters, Repair or Replace</t>
+          <t>What Are Fascias and Soffits on a House?</t>
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Concrete Finlock Gutters, Repair or Replace</t>
+          <t>What Are Fascias and Soffits on a House?</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); three cost tables (by property type, additional costs, lifespan) from the client's records; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
+          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); comparison or step table; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
@@ -4034,14 +4034,14 @@
       </c>
       <c r="N53" s="2" t="inlineStr">
         <is>
-          <t>240 UK searches a month across 4 searches (concrete gutter replacement cost 70; concrete gutter repair 70; finlock gutter removal cost 50; finlock gutter repair 50). Overlap test against /gutter-replacement/ before writing</t>
+          <t>4,120 UK searches a month across 19 searches (what are soffits and fascias 1300; what are fascias on a house 590; fascia vs soffit 320; what are soffits on a house 320). Overlap test passed: 0% vs "fascias and soffits manchester" (/fascias-and-soffits/)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>/blog/what-are-fascias-and-soffits/</t>
+          <t>/blog/leaking-gutter-joint/</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -4059,20 +4059,20 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Launch, after the overlap test</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>What Are Fascias and Soffits on a House?</t>
+          <t>How to Fix a Leaking Gutter Joint | Manchester Gutters</t>
         </is>
       </c>
       <c r="G54" s="2" t="n">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>What Are Fascias and Soffits on a House?</t>
+          <t>How to Fix a Leaking Gutter Joint</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
@@ -4102,14 +4102,14 @@
       </c>
       <c r="N54" s="2" t="inlineStr">
         <is>
-          <t>4,120 UK searches a month across 19 searches (what are soffits and fascias 1300; what are fascias on a house 590; fascia vs soffit 320; what are soffits on a house 320). Overlap test against /fascias-and-soffits/ before writing</t>
+          <t>2,410 UK searches a month across 16 searches (gutter leaking at joint 1000; sealing gutter joints 390; how to fix a leaking gutter joint 260; fix leaking gutter joint 170). Overlap test passed: 30% vs "gutter leaking" (/blog/why-is-my-gutter-leaking/)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>/blog/leaking-gutter-joint/</t>
+          <t>/blog/why-is-my-gutter-leaking/</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -4127,20 +4127,20 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Launch, after the overlap test</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>How to Fix a Leaking Gutter Joint | Manchester Gutters</t>
+          <t>Why Is My Gutter Leaking and How to Fix It</t>
         </is>
       </c>
       <c r="G55" s="2" t="n">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>How to Fix a Leaking Gutter Joint</t>
+          <t>Why Is My Gutter Leaking and How to Fix It</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
@@ -4170,14 +4170,14 @@
       </c>
       <c r="N55" s="2" t="inlineStr">
         <is>
-          <t>2,410 UK searches a month across 16 searches (gutter leaking at joint 1000; sealing gutter joints 390; how to fix a leaking gutter joint 260; fix leaking gutter joint 170). Overlap test against /gutter-repairs/ before writing</t>
+          <t>1,600 UK searches a month across 13 searches (gutter leaking 480; gutter leak repairs 480; how to fix a leaking gutter 210; sealing gutter leaks 140). Overlap test passed: 0% vs "gutter repairs manchester" (/gutter-repairs/)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>/blog/why-is-my-gutter-leaking/</t>
+          <t>/blog/blocked-downpipe/</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -4200,15 +4200,15 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Why Is My Gutter Leaking and How to Fix It</t>
+          <t>Blocked or Leaking Downpipe? What to Do | Manchester Gutters</t>
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Why Is My Gutter Leaking and How to Fix It</t>
+          <t>Blocked or Leaking Downpipe? What to Do</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
@@ -4238,14 +4238,14 @@
       </c>
       <c r="N56" s="2" t="inlineStr">
         <is>
-          <t>1,600 UK searches a month across 13 searches (gutter leaking 480; gutter leak repairs 480; how to fix a leaking gutter 210; sealing gutter leaks 140). Overlap test against /gutter-repairs/ before writing</t>
+          <t>990 UK searches a month across 11 searches (downpipe blocked 260; blocked downpipe from gutter 210; how to unblock a downpipe 110; downpipe leaking 90). Overlap test against /downpipes/ before writing</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>/blog/blocked-downpipe/</t>
+          <t>/blog/rotten-fascia-boards/</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -4268,15 +4268,15 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Blocked or Leaking Downpipe? What to Do | Manchester Gutters</t>
+          <t>Rotten Fascia Boards, Repair or Replace?</t>
         </is>
       </c>
       <c r="G57" s="2" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Blocked or Leaking Downpipe? What to Do</t>
+          <t>Rotten Fascia Boards, Repair or Replace?</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
@@ -4306,14 +4306,14 @@
       </c>
       <c r="N57" s="2" t="inlineStr">
         <is>
-          <t>990 UK searches a month across 11 searches (downpipe blocked 260; blocked downpipe from gutter 210; how to unblock a downpipe 110; downpipe leaking 90). Overlap test against /downpipes/ before writing</t>
+          <t>980 UK searches a month across 14 searches (fixing soffits and fascias 170; how to fit fascia boards 140; how to replace fascia and soffit 110; how to install fascia boards 90). Folded in as sections: signs fascia needs replacing. Overlap test against /fascias-and-soffits/ before writing</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>/blog/rotten-fascia-boards/</t>
+          <t>/blog/box-gutter-leaking/</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -4336,15 +4336,15 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Rotten Fascia Boards, Repair or Replace?</t>
+          <t>Leaking Box Gutters and Conservatory Gutters</t>
         </is>
       </c>
       <c r="G58" s="2" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Rotten Fascia Boards, Repair or Replace?</t>
+          <t>Leaking Box Gutters and Conservatory Gutters</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
@@ -4374,14 +4374,14 @@
       </c>
       <c r="N58" s="2" t="inlineStr">
         <is>
-          <t>980 UK searches a month across 14 searches (fixing soffits and fascias 170; how to fit fascia boards 140; how to replace fascia and soffit 110; how to install fascia boards 90). Folded in as sections: signs fascia needs replacing. Overlap test against /fascias-and-soffits/ before writing</t>
+          <t>380 UK searches a month across 5 searches (conservatory box gutter leaking 140; what are box gutters 90; fixing box gutters 70; box gutter sizes 50). Overlap test against /gutter-repairs/ before writing</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>/blog/box-gutter-leaking/</t>
+          <t>/blog/gutters-overflowing/</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -4404,15 +4404,15 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Leaking Box Gutters and Conservatory Gutters</t>
+          <t>Why Are My Gutters Overflowing? | Manchester Gutters</t>
         </is>
       </c>
       <c r="G59" s="2" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Leaking Box Gutters and Conservatory Gutters</t>
+          <t>Why Are My Gutters Overflowing?</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
@@ -4442,14 +4442,14 @@
       </c>
       <c r="N59" s="2" t="inlineStr">
         <is>
-          <t>380 UK searches a month across 5 searches (conservatory box gutter leaking 140; what are box gutters 90; fixing box gutters 70; box gutter sizes 50). Overlap test against /gutter-repairs/ before writing</t>
+          <t>340 UK searches a month across 3 searches (gutters overflowing 260; gutter overflowing in heavy rain 70; why are my gutters overflowing 10). Overlap test against /gutter-repairs/ before writing</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>/blog/gutters-overflowing/</t>
+          <t>/blog/gutter-fall-and-bracket-spacing/</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -4472,15 +4472,15 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Why Are My Gutters Overflowing? | Manchester Gutters</t>
+          <t>Gutter Brackets and Fall Explained | Manchester Gutters</t>
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Why Are My Gutters Overflowing?</t>
+          <t>Gutter Brackets and Fall Explained</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
@@ -4510,14 +4510,14 @@
       </c>
       <c r="N60" s="2" t="inlineStr">
         <is>
-          <t>340 UK searches a month across 3 searches (gutters overflowing 260; gutter overflowing in heavy rain 70; why are my gutters overflowing 10). Overlap test against /gutter-repairs/ before writing</t>
+          <t>2,480 UK searches a month across 20 searches (gutter brackets rise and fall 590; fall for guttering 480; types of gutter brackets 170; guttering fall per metre 140). Overlap test against /gutter-replacement/ before writing</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>/blog/gutter-fall-and-bracket-spacing/</t>
+          <t>/blog/how-to-replace-guttering/</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -4540,15 +4540,15 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Gutter Brackets and Fall Explained | Manchester Gutters</t>
+          <t>How to Replace Guttering Step by Step | Manchester Gutters</t>
         </is>
       </c>
       <c r="G61" s="2" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Gutter Brackets and Fall Explained</t>
+          <t>How to Replace Guttering Step by Step</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
@@ -4578,14 +4578,14 @@
       </c>
       <c r="N61" s="2" t="inlineStr">
         <is>
-          <t>2,480 UK searches a month across 20 searches (gutter brackets rise and fall 590; fall for guttering 480; types of gutter brackets 170; guttering fall per metre 140). Overlap test against /gutter-replacement/ before writing</t>
+          <t>1,290 UK searches a month across 14 searches (how to replace guttering 480; how to fit guttering 210; how to fix guttering 170; how to cut guttering 170). Folded in as sections: tools for fitting guttering, gutter installation mistakes. Sister site: Munster step-by-step installation guide: 68 clicks. Overlap test against /gutter-replacement/ before writing</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>/blog/how-to-replace-guttering/</t>
+          <t>/blog/are-gutter-guards-worth-it/</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -4608,15 +4608,15 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>How to Replace Guttering Step by Step | Manchester Gutters</t>
+          <t>Gutter Guards, Are They Worth Fitting? | Manchester Gutters</t>
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>How to Replace Guttering Step by Step</t>
+          <t>Gutter Guards, Are They Worth Fitting?</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
@@ -4646,14 +4646,14 @@
       </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>1,290 UK searches a month across 14 searches (how to replace guttering 480; how to fit guttering 210; how to fix guttering 170; how to cut guttering 170). Folded in as sections: tools for fitting guttering, gutter installation mistakes. Sister site: Munster step-by-step installation guide: 68 clicks. Overlap test against /gutter-replacement/ before writing</t>
+          <t>350 UK searches a month across 6 searches (best gutter guards 170; cost of gutter guards 50; are gutter guards worth it 40; what gutter guard is best 30). Overlap test against /gutter-replacement/ before writing</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>/blog/are-gutter-guards-worth-it/</t>
+          <t>/blog/rogue-roofers/</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -4676,15 +4676,15 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Gutter Guards, Are They Worth Fitting? | Manchester Gutters</t>
+          <t>How to Spot a Rogue Roofer and Hire Safely</t>
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Gutter Guards, Are They Worth Fitting?</t>
+          <t>How to Spot a Rogue Roofer and Hire Safely</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
@@ -4714,23 +4714,23 @@
       </c>
       <c r="N63" s="2" t="inlineStr">
         <is>
-          <t>350 UK searches a month across 6 searches (best gutter guards 170; cost of gutter guards 50; are gutter guards worth it 40; what gutter guard is best 30). Overlap test against /gutter-replacement/ before writing</t>
+          <t>280 UK searches a month across 6 searches (roofing scams 90; cowboy roofers 90; rogue roofers 40; roofing scams uk 30). Folded in as sections: how to complain about a builder. Sister site: Munster "Irish roofer scams": 72 clicks</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>/blog/rogue-roofers/</t>
+          <t>/blog/</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Article: pillar</t>
+          <t>Blog index</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
@@ -4739,62 +4739,58 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Launch, after the overlap test</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>How to Spot a Rogue Roofer and Hire Safely</t>
+          <t>Guttering Guides and Costs | Manchester Gutters</t>
         </is>
       </c>
       <c r="G64" s="2" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>How to Spot a Rogue Roofer and Hire Safely</t>
+          <t>Guttering guides</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>1,000-1,800</t>
+          <t>200-400</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>Breadcrumb + meta; photo; 40-60-word answer; at a glance bullets; contents list (H2 anchors); Read next; question H2s (60%+); comparison or step table; case/review/video if records; who to hire; guarantees; FAQ 10-12; sources and further reading; related cards; CTA + form</t>
+          <t>Groups by topic; 20 cards then pages</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>blog index; hub guide cards</t>
+          <t>nav</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>services (3-5 in prose); the place hub; Read next 3-4; primary sources</t>
+          <t>every article</t>
         </is>
       </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>BlogPosting, BreadcrumbList, FAQPage</t>
-        </is>
-      </c>
-      <c r="N64" s="2" t="inlineStr">
-        <is>
-          <t>280 UK searches a month across 6 searches (roofing scams 90; cowboy roofers 90; rogue roofers 40; roofing scams uk 30). Folded in as sections: how to complain about a builder. Sister site: Munster "Irish roofer scams": 72 clicks</t>
-        </is>
-      </c>
+          <t>CollectionPage, BreadcrumbList</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>/blog/</t>
+          <t>/reviews/</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Blog index</t>
+          <t>Proof</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4807,45 +4803,45 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>When records exist</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Guttering Guides and Costs | Manchester Gutters</t>
+          <t>Manchester Gutters Reviews and Ratings</t>
         </is>
       </c>
       <c r="G65" s="2" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Guttering guides</t>
+          <t>Manchester Gutters Reviews and Ratings</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>200-400</t>
+          <t>as records allow</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>Groups by topic; 20 cards then pages</t>
+          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>nav</t>
+          <t>nav; footer; towns and services (1 in prose)</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>every article</t>
+          <t>issuers (Google profile, memberships)</t>
         </is>
       </c>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>CollectionPage, BreadcrumbList</t>
+          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
         </is>
       </c>
       <c r="N65" s="2" t="inlineStr"/>
@@ -4853,7 +4849,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>/reviews/</t>
+          <t>/case-studies/</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -4876,15 +4872,15 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Manchester Gutters Reviews and Ratings</t>
+          <t>Case Studies | Manchester Gutters</t>
         </is>
       </c>
       <c r="G66" s="2" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Manchester Gutters Reviews and Ratings</t>
+          <t>Case Studies</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -4917,7 +4913,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>/case-studies/</t>
+          <t>/price-guide/</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -4940,15 +4936,15 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Case Studies | Manchester Gutters</t>
+          <t>Guttering Price Guide | Manchester Gutters</t>
         </is>
       </c>
       <c r="G67" s="2" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Case Studies</t>
+          <t>Guttering Price Guide</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -4981,7 +4977,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>/price-guide/</t>
+          <t>/gallery/</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -5004,15 +5000,15 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Guttering Price Guide | Manchester Gutters</t>
+          <t>Gallery of Recent Jobs | Manchester Gutters</t>
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Guttering Price Guide</t>
+          <t>Gallery of Recent Jobs</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
@@ -5045,12 +5041,12 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>/gallery/</t>
+          <t>/about/</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Proof</t>
+          <t>Company</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -5063,45 +5059,45 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>When records exist</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Gallery of Recent Jobs | Manchester Gutters</t>
+          <t>About Manchester Gutters | Local Guttering Team</t>
         </is>
       </c>
       <c r="G69" s="2" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>Gallery of Recent Jobs</t>
+          <t>About Manchester Gutters</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>as records allow</t>
+          <t>600-1,200</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>Records only (exact quotes, dated, with area; or case cards, photos, price tables); check-it-yourself links; CTA + form</t>
+          <t>Named people, credentials table, contact by area, map after consent</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>nav; footer; towns and services (1 in prose)</t>
+          <t>nav; footer</t>
         </is>
       </c>
       <c r="L69" s="2" t="inlineStr">
         <is>
-          <t>issuers (Google profile, memberships)</t>
+          <t>nav only</t>
         </is>
       </c>
       <c r="M69" s="2" t="inlineStr">
         <is>
-          <t>Organization reference; Review/AggregateRating only where shown; ImageGallery</t>
+          <t>AboutPage / ContactPage + Organization reference</t>
         </is>
       </c>
       <c r="N69" s="2" t="inlineStr"/>
@@ -5109,7 +5105,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>/about/</t>
+          <t>/contact/</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -5132,15 +5128,15 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>About Manchester Gutters | Local Guttering Team</t>
+          <t>Contact Manchester Gutters | Free Guttering Quotes</t>
         </is>
       </c>
       <c r="G70" s="2" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>About Manchester Gutters</t>
+          <t>Contact Manchester Gutters</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
@@ -5173,12 +5169,12 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>/contact/</t>
+          <t>/privacy-policy/</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Company</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -5196,25 +5192,25 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Contact Manchester Gutters | Free Guttering Quotes</t>
+          <t>Privacy Policy | Manchester Gutters</t>
         </is>
       </c>
       <c r="G71" s="2" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Contact Manchester Gutters</t>
+          <t>Privacy Policy</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>600-1,200</t>
+          <t>as needed</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>Named people, credentials table, contact by area, map after consent</t>
+          <t>What the site really does</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr">
@@ -5229,7 +5225,7 @@
       </c>
       <c r="M71" s="2" t="inlineStr">
         <is>
-          <t>AboutPage / ContactPage + Organization reference</t>
+          <t>WebPage</t>
         </is>
       </c>
       <c r="N71" s="2" t="inlineStr"/>
@@ -5237,7 +5233,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>/privacy-policy/</t>
+          <t>/cookie-policy/</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -5260,15 +5256,15 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Privacy Policy | Manchester Gutters</t>
+          <t>Cookie Policy | Manchester Gutters</t>
         </is>
       </c>
       <c r="G72" s="2" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>Privacy Policy</t>
+          <t>Cookie Policy</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
@@ -5301,71 +5297,77 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>/cookie-policy/</t>
+          <t>/404</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Legal</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="n">
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Non-indexable</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D73" s="2" t="inlineStr">
-        <is>
-          <t>Indexable</t>
-        </is>
-      </c>
-      <c r="E73" s="2" t="inlineStr">
-        <is>
-          <t>Launch</t>
-        </is>
-      </c>
-      <c r="F73" s="2" t="inlineStr">
-        <is>
-          <t>Cookie Policy | Manchester Gutters</t>
-        </is>
-      </c>
-      <c r="G73" s="2" t="n">
-        <v>34</v>
-      </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Cookie Policy</t>
+          <t>–</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>as needed</t>
+          <t>–</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>What the site really does</t>
+          <t>–</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>nav; footer</t>
+          <t>–</t>
         </is>
       </c>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t>nav only</t>
+          <t>–</t>
         </is>
       </c>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>WebPage</t>
-        </is>
-      </c>
-      <c r="N73" s="2" t="inlineStr"/>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr">
+        <is>
+          <t>served with HTTP status 404</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>/404</t>
+          <t>/sitemap.xml</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -5428,14 +5430,14 @@
       </c>
       <c r="N74" s="2" t="inlineStr">
         <is>
-          <t>served with HTTP status 404</t>
+          <t>indexable pages only; real lastmod dates</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>/sitemap.xml</t>
+          <t>/robots.txt</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -5498,14 +5500,14 @@
       </c>
       <c r="N75" s="2" t="inlineStr">
         <is>
-          <t>indexable pages only; real lastmod dates</t>
+          <t>allows the AI search crawlers; points to the sitemap</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>/robots.txt</t>
+          <t>/llms.txt</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -5568,82 +5570,12 @@
       </c>
       <c r="N76" s="2" t="inlineStr">
         <is>
-          <t>allows the AI search crawlers; points to the sitemap</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>/llms.txt</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>Utility</t>
-        </is>
-      </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
-        <is>
-          <t>Non-indexable</t>
-        </is>
-      </c>
-      <c r="E77" s="2" t="inlineStr">
-        <is>
-          <t>Launch</t>
-        </is>
-      </c>
-      <c r="F77" s="2" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G77" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H77" s="2" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I77" s="2" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="J77" s="2" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="K77" s="2" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="L77" s="2" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M77" s="2" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N77" s="2" t="inlineStr">
-        <is>
           <t>public facts only, from the facts file</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N77"/>
+  <autoFilter ref="A1:N76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: sync site-content skill after audit-content#626
Overlap test results for the other eight Manchester articles (all stand),
the rebuilt URL map and site tree, and the updated topic-research note.
Copy identical to audit-content site-content/manchester-overlap-tests-2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016DXh5ATFKvUL6hqSuDkrz5
</commit_message>
<xml_diff>
--- a/.claude/skills/site-content/assets/manchester-gutters-url-map.xlsx
+++ b/.claude/skills/site-content/assets/manchester-gutters-url-map.xlsx
@@ -3923,7 +3923,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Launch, after the overlap test</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3966,7 +3966,7 @@
       </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>240 UK searches a month across 4 searches (concrete gutter replacement cost 70; concrete gutter repair 70; finlock gutter removal cost 50; finlock gutter repair 50). Overlap test against /gutter-replacement/ before writing</t>
+          <t>240 UK searches a month across 4 searches (concrete gutter replacement cost 70; concrete gutter repair 70; finlock gutter removal cost 50; finlock gutter repair 50). Overlap test passed: 20% vs "gutter replacement manchester" (/gutter-replacement/); 40% vs "gutter replacement cost" (/blog/gutter-replacement-cost/)</t>
         </is>
       </c>
     </row>
@@ -4195,7 +4195,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Launch, after the overlap test</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -4238,7 +4238,7 @@
       </c>
       <c r="N56" s="2" t="inlineStr">
         <is>
-          <t>990 UK searches a month across 11 searches (downpipe blocked 260; blocked downpipe from gutter 210; how to unblock a downpipe 110; downpipe leaking 90). Overlap test against /downpipes/ before writing</t>
+          <t>990 UK searches a month across 11 searches (downpipe blocked 260; blocked downpipe from gutter 210; how to unblock a downpipe 110; downpipe leaking 90). Overlap test passed: 0% vs "downpipe repairs manchester" (/downpipes/)</t>
         </is>
       </c>
     </row>
@@ -4263,7 +4263,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Launch, after the overlap test</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -4306,7 +4306,7 @@
       </c>
       <c r="N57" s="2" t="inlineStr">
         <is>
-          <t>980 UK searches a month across 14 searches (fixing soffits and fascias 170; how to fit fascia boards 140; how to replace fascia and soffit 110; how to install fascia boards 90). Folded in as sections: signs fascia needs replacing. Overlap test against /fascias-and-soffits/ before writing</t>
+          <t>980 UK searches a month across 14 searches (fixing soffits and fascias 170; how to fit fascia boards 140; how to replace fascia and soffit 110; how to install fascia boards 90). Folded in as sections: signs fascia needs replacing. Overlap test passed: 10% vs "fascias and soffits manchester" (/fascias-and-soffits/); 10% vs "fascia and soffit replacement cost" (/blog/fascia-and-soffit-replacement-cost/)</t>
         </is>
       </c>
     </row>
@@ -4331,7 +4331,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Launch, after the overlap test</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -4374,7 +4374,7 @@
       </c>
       <c r="N58" s="2" t="inlineStr">
         <is>
-          <t>380 UK searches a month across 5 searches (conservatory box gutter leaking 140; what are box gutters 90; fixing box gutters 70; box gutter sizes 50). Overlap test against /gutter-repairs/ before writing</t>
+          <t>380 UK searches a month across 5 searches (conservatory box gutter leaking 140; what are box gutters 90; fixing box gutters 70; box gutter sizes 50). Overlap test passed: 0% vs "gutter repairs manchester" (/gutter-repairs/); 10% vs "gutter leaking" (/blog/why-is-my-gutter-leaking/)</t>
         </is>
       </c>
     </row>
@@ -4399,7 +4399,7 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Launch, after the overlap test</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -4442,7 +4442,7 @@
       </c>
       <c r="N59" s="2" t="inlineStr">
         <is>
-          <t>340 UK searches a month across 3 searches (gutters overflowing 260; gutter overflowing in heavy rain 70; why are my gutters overflowing 10). Overlap test against /gutter-repairs/ before writing</t>
+          <t>340 UK searches a month across 3 searches (gutters overflowing 260; gutter overflowing in heavy rain 70; why are my gutters overflowing 10). Overlap test passed: 0% vs "gutter repairs manchester" (/gutter-repairs/); 10% vs "gutter leaking" (/blog/why-is-my-gutter-leaking/)</t>
         </is>
       </c>
     </row>
@@ -4467,7 +4467,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Launch, after the overlap test</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -4510,7 +4510,7 @@
       </c>
       <c r="N60" s="2" t="inlineStr">
         <is>
-          <t>2,480 UK searches a month across 20 searches (gutter brackets rise and fall 590; fall for guttering 480; types of gutter brackets 170; guttering fall per metre 140). Overlap test against /gutter-replacement/ before writing</t>
+          <t>2,480 UK searches a month across 20 searches (gutter brackets rise and fall 590; fall for guttering 480; types of gutter brackets 170; guttering fall per metre 140). Overlap test passed: 0% vs "gutter replacement manchester" (/gutter-replacement/); 0% vs "how to replace guttering" (/blog/how-to-replace-guttering/)</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4535,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Launch, after the overlap test</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -4578,7 +4578,7 @@
       </c>
       <c r="N61" s="2" t="inlineStr">
         <is>
-          <t>1,290 UK searches a month across 14 searches (how to replace guttering 480; how to fit guttering 210; how to fix guttering 170; how to cut guttering 170). Folded in as sections: tools for fitting guttering, gutter installation mistakes. Sister site: Munster step-by-step installation guide: 68 clicks. Overlap test against /gutter-replacement/ before writing</t>
+          <t>1,290 UK searches a month across 14 searches (how to replace guttering 480; how to fit guttering 210; how to fix guttering 170; how to cut guttering 170). Folded in as sections: tools for fitting guttering, gutter installation mistakes. Sister site: Munster step-by-step installation guide: 68 clicks. Overlap test passed: 0% vs "gutter replacement manchester" (/gutter-replacement/); 0% vs "gutter replacement cost" (/blog/gutter-replacement-cost/)</t>
         </is>
       </c>
     </row>
@@ -4603,7 +4603,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Launch, after the overlap test</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -4646,7 +4646,7 @@
       </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>350 UK searches a month across 6 searches (best gutter guards 170; cost of gutter guards 50; are gutter guards worth it 40; what gutter guard is best 30). Overlap test against /gutter-replacement/ before writing</t>
+          <t>350 UK searches a month across 6 searches (best gutter guards 170; cost of gutter guards 50; are gutter guards worth it 40; what gutter guard is best 30). Overlap test passed: 0% vs "gutter replacement manchester" (/gutter-replacement/)</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Launch, after the overlap test</t>
+          <t>Launch</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">

</xml_diff>